<commit_message>
implemented stronghold retaliation, energy drops, and csv controlled enemy spawning
repositioned the energy counter below the defender toolbar to stop overlapping
added stronghold retaliation damage against melee and crusher enemies.
added retaliation damage stat config in excel csv
25% for defeated enemies to drop an energy ball worth 20 energy (for now)
updated enemy ts to trigger energy drops when enemies are defeated
configured spawn probabilities: 45%melee, 45% ranged, 10% crusher (for now)
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView/>
+    <workbookView firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>enemy_id</t>
   </si>
@@ -96,12 +96,21 @@
     <t>pickup_lifetime_ms</t>
   </si>
   <si>
+    <t>enemy_drop_chance</t>
+  </si>
+  <si>
+    <t>enemy_drop_value</t>
+  </si>
+  <si>
     <t>starting_health</t>
   </si>
   <si>
     <t>melee_attack_interval_ms</t>
   </si>
   <si>
+    <t>retaliation_damage</t>
+  </si>
+  <si>
     <t>first_enemy_delay_ms</t>
   </si>
   <si>
@@ -112,6 +121,9 @@
   </si>
   <si>
     <t>ranged_spawn_probability</t>
+  </si>
+  <si>
+    <t>crusher_spawn_probability</t>
   </si>
 </sst>
 </file>
@@ -167,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -176,6 +188,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,7 +484,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{993BD573-A344-32E8-D178-FC57EF4915D5}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A2FE8D48-F8C8-45CA-4BD3-F030A7927EC7}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -600,7 +613,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9A3A3937-C90F-7A08-6438-305329E84418}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BAC54AC8-45A8-01B8-8646-6DB2A3BBFBB6}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -647,7 +660,7 @@
         <v>300</v>
       </c>
       <c r="C2" s="1">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1">
         <v>100</v>
@@ -725,7 +738,7 @@
         <v>300</v>
       </c>
       <c r="C5" s="2">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2">
         <v>200</v>
@@ -738,6 +751,9 @@
       </c>
       <c r="G5" s="2">
         <v>300</v>
+      </c>
+      <c r="H5" s="4">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -753,7 +769,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{37E1B0F7-1571-3948-16A8-2C7FBEBBA918}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3F832736-7616-8D68-FFDF-CB585BF12E88}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -806,6 +822,22 @@
       </c>
       <c r="B6" s="1">
         <v>15000</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="4">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="4">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -821,7 +853,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{769776D8-92D8-1248-4BC2-251BC106C7A8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{80D8D744-3F3B-8A4E-FEE8-A6A0C1A6BA88}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -838,7 +870,7 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -846,10 +878,18 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="4">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -865,7 +905,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{68161718-49B3-8D78-0DEE-1244F314FEB9}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5AA6DB8F-C198-16DF-CD08-DD4B680E82B1}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -882,7 +922,7 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1">
         <v>20000</v>
@@ -890,7 +930,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B3" s="1">
         <v>15000</v>
@@ -898,18 +938,26 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B4" s="1">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B5" s="1">
-        <v>0.5</v>
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adjusted some stat values
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView firstSheet="2" activeTab="4"/>
+    <workbookView firstSheet="2" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -179,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -188,7 +188,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,7 +483,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A2FE8D48-F8C8-45CA-4BD3-F030A7927EC7}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{77209764-9143-BACE-CC26-78DE0F7778AD}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -613,7 +612,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BAC54AC8-45A8-01B8-8646-6DB2A3BBFBB6}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3C424B91-994B-81F6-0B0D-0FEA35CD8686}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -752,7 +751,7 @@
       <c r="G5" s="2">
         <v>300</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="2">
         <v>20</v>
       </c>
     </row>
@@ -769,7 +768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3F832736-7616-8D68-FFDF-CB585BF12E88}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E2A3EC32-99C9-7528-26E8-227872FC6008}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -825,18 +824,18 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="4">
-        <v>0.25</v>
+      <c r="B7" s="2">
+        <v>0.4</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <v>20</v>
       </c>
     </row>
@@ -853,7 +852,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{80D8D744-3F3B-8A4E-FEE8-A6A0C1A6BA88}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0E011E58-0FAA-9CD2-B4C9-BFCA2D2F425D}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -885,10 +884,10 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <v>50</v>
       </c>
     </row>
@@ -905,7 +904,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5AA6DB8F-C198-16DF-CD08-DD4B680E82B1}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CDB34B18-4166-034B-0648-5D0D8D2B8D65}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -933,7 +932,7 @@
         <v>32</v>
       </c>
       <c r="B3" s="1">
-        <v>15000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
@@ -941,7 +940,7 @@
         <v>33</v>
       </c>
       <c r="B4" s="1">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -949,15 +948,15 @@
         <v>34</v>
       </c>
       <c r="B5" s="1">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="4">
-        <v>0.1</v>
+      <c r="B6" s="2">
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implement level 1 and level 2 wave progression
implemented excel config wave counts and enemy limits
completed level 1 with one wave of 3 melee enemies (for now)
completed level 2 with two waves of 3 and 5 melee enemies (for now)
updated wavemanager to track wave progression and level completion
fixed enemy spawning to stop when the wave limit is reached
updated wave counter to display the correct wave number
connected the level complete screen to the next level button
fixed csv configs issues affecting wave settings
level 1 and level progression works
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView firstSheet="2" activeTab="2"/>
+    <workbookView firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>enemy_id</t>
   </si>
@@ -124,6 +124,15 @@
   </si>
   <si>
     <t>crusher_spawn_probability</t>
+  </si>
+  <si>
+    <t>level_1_wave_count</t>
+  </si>
+  <si>
+    <t>starting_enemies_per_wave</t>
+  </si>
+  <si>
+    <t>level_2_wave_count</t>
   </si>
 </sst>
 </file>
@@ -179,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -188,6 +197,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -483,7 +493,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{77209764-9143-BACE-CC26-78DE0F7778AD}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{EA814938-8698-C791-D2D5-652007DECC35}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -612,7 +622,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3C424B91-994B-81F6-0B0D-0FEA35CD8686}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DF2D5748-E7E8-DE4D-F538-C562273C2178}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -768,7 +778,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E2A3EC32-99C9-7528-26E8-227872FC6008}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{30B4F6B8-947C-4948-C02C-D1C8D694E1B8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -852,7 +862,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0E011E58-0FAA-9CD2-B4C9-BFCA2D2F425D}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BB92029B-C056-4DB8-C6D8-9749C24E108F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -904,11 +914,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CDB34B18-4166-034B-0648-5D0D8D2B8D65}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{40939ABD-8C68-D5DB-3692-E0EF3B5955EF}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="23.28125" customWidth="1"/>
+    <col min="1" max="1" width="24.57421875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -940,7 +950,7 @@
         <v>33</v>
       </c>
       <c r="B4" s="1">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -948,7 +958,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="1">
-        <v>0.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -956,7 +966,31 @@
         <v>35</v>
       </c>
       <c r="B6" s="2">
-        <v>0.05</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="4">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
5 level progression system and enemy spawning
added config wave counts for wave 3,4,5
updated wavemanager to allow progression across all 5 levels
melee enemy only spawns in level 1
ranged enemy introduced in level 2
crusher enemy introduced in level 3
guaranteed first appearence (ranged, crusher enemy) for their level
fixed tracking in wavemanager
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>enemy_id</t>
   </si>
@@ -133,6 +133,15 @@
   </si>
   <si>
     <t>level_2_wave_count</t>
+  </si>
+  <si>
+    <t>level_3_wave_count</t>
+  </si>
+  <si>
+    <t>level_4_wave_count</t>
+  </si>
+  <si>
+    <t>level_5_wave_count</t>
   </si>
 </sst>
 </file>
@@ -493,7 +502,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{EA814938-8698-C791-D2D5-652007DECC35}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{F46068BC-942A-CC08-80DB-D218E45AA0A7}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -622,7 +631,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DF2D5748-E7E8-DE4D-F538-C562273C2178}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D68FBFFB-7F28-7E08-8398-E869543F240F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -778,7 +787,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{30B4F6B8-947C-4948-C02C-D1C8D694E1B8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B8837308-4108-4A08-3A78-269F371CBD11}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -862,7 +871,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BB92029B-C056-4DB8-C6D8-9749C24E108F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A116588D-0028-1834-2F81-495E922C2226}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -914,7 +923,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{40939ABD-8C68-D5DB-3692-E0EF3B5955EF}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4B1956F8-21A7-D23B-B668-9107B445F96D}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -950,7 +959,7 @@
         <v>33</v>
       </c>
       <c r="B4" s="1">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -958,7 +967,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="1">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -966,32 +975,59 @@
         <v>35</v>
       </c>
       <c r="B6" s="2">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <v>2</v>
       </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="4"/>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>

<commit_message>
implement excel configurable wave budget system
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>enemy_id</t>
   </si>
@@ -142,6 +142,51 @@
   </si>
   <si>
     <t>level_5_wave_count</t>
+  </si>
+  <si>
+    <t>melee_wave_cost</t>
+  </si>
+  <si>
+    <t>ranged_wave_cost</t>
+  </si>
+  <si>
+    <t>crusher_wave_cost</t>
+  </si>
+  <si>
+    <t>level_1_wave_1_budget</t>
+  </si>
+  <si>
+    <t>level_2_wave_1_budget</t>
+  </si>
+  <si>
+    <t>level_2_wave_2_budget</t>
+  </si>
+  <si>
+    <t>level_3_wave_1_budget</t>
+  </si>
+  <si>
+    <t>level_3_wave_2_budget</t>
+  </si>
+  <si>
+    <t>level_3_wave_3_budget</t>
+  </si>
+  <si>
+    <t>level_4_wave_1_budget</t>
+  </si>
+  <si>
+    <t>level_4_wave_2_budget</t>
+  </si>
+  <si>
+    <t>level_4_wave_3_budget</t>
+  </si>
+  <si>
+    <t>level_5_wave_1_budget</t>
+  </si>
+  <si>
+    <t>level_5_wave_2_budget</t>
+  </si>
+  <si>
+    <t>level_5_wave_3_budget</t>
   </si>
 </sst>
 </file>
@@ -502,7 +547,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{F46068BC-942A-CC08-80DB-D218E45AA0A7}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DD4A6DF8-0D16-269D-FF59-B7DD3A4B4E93}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -631,7 +676,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D68FBFFB-7F28-7E08-8398-E869543F240F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AB5948EA-2088-2D6A-0291-BCC513850737}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -787,7 +832,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B8837308-4108-4A08-3A78-269F371CBD11}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AB816F12-9811-1DCB-B958-AC70F6A4B326}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -871,7 +916,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A116588D-0028-1834-2F81-495E922C2226}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{045C0E58-7773-ACF5-507B-BF23312259BA}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -923,7 +968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4B1956F8-21A7-D23B-B668-9107B445F96D}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{35709781-6218-E278-DD58-6CC7BBF2DD3A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1027,7 +1072,124 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="B13" s="4"/>
+      <c r="A13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="4">
+        <v>110</v>
+      </c>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>

<commit_message>
added new defender cryogunner
added two new files for the defender called cryogunner, he slows down enemies
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView firstSheet="2" activeTab="4"/>
+    <workbookView activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>enemy_id</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>dualbarrel</t>
+  </si>
+  <si>
+    <t>cryogunner</t>
   </si>
   <si>
     <t>setting</t>
@@ -547,7 +550,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DD4A6DF8-0D16-269D-FF59-B7DD3A4B4E93}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3204F838-D798-3BA8-BBE8-E62C7E3B17F8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -676,7 +679,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AB5948EA-2088-2D6A-0291-BCC513850737}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{81A3A98D-2348-6328-1256-C48FF09DB968}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -819,6 +822,32 @@
         <v>20</v>
       </c>
     </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="4">
+        <v>300</v>
+      </c>
+      <c r="C6" s="4">
+        <v>20</v>
+      </c>
+      <c r="D6" s="4">
+        <v>175</v>
+      </c>
+      <c r="E6" s="4">
+        <v>10000</v>
+      </c>
+      <c r="F6" s="4">
+        <v>100</v>
+      </c>
+      <c r="G6" s="4">
+        <v>300</v>
+      </c>
+      <c r="H6" s="4">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -832,7 +861,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AB816F12-9811-1DCB-B958-AC70F6A4B326}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CA10F698-A2B8-E168-D458-09A5F3493698}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -841,15 +870,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -857,7 +886,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -865,7 +894,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -873,7 +902,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -881,7 +910,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -889,7 +918,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -897,7 +926,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -916,7 +945,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{045C0E58-7773-ACF5-507B-BF23312259BA}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CF557CBB-C3F8-17D8-2DFD-001EE8494571}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -925,15 +954,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -941,7 +970,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -949,7 +978,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -968,7 +997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{35709781-6218-E278-DD58-6CC7BBF2DD3A}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{36E36338-5F88-45FD-39F8-DC72C5B9A5E8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -977,15 +1006,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1">
         <v>20000</v>
@@ -993,7 +1022,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B3" s="1">
         <v>5000</v>
@@ -1001,7 +1030,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1009,7 +1038,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1017,7 +1046,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1025,7 +1054,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1033,7 +1062,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1041,153 +1070,153 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="4">
+      <c r="A10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="2">
         <v>40</v>
       </c>
-      <c r="B11" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" s="4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="4">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="4">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" s="4">
-        <v>40</v>
-      </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B20" s="4">
+      <c r="A20" s="2" t="s">
         <v>50</v>
       </c>
+      <c r="B20" s="2">
+        <v>50</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="2">
         <v>50</v>
       </c>
-      <c r="B21" s="4">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="4">
-        <v>50</v>
-      </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B23" s="4">
+      <c r="A23" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="2">
         <v>65</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="4">
+      <c r="A24" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="2">
         <v>80</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B25" s="4">
+      <c r="A25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="2">
         <v>70</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" s="4">
+      <c r="A26" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="2">
         <v>90</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" s="4">
+      <c r="A27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B27" s="2">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added passive energy accumalation as the progression happens using spreadsheet
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView activeTab="1"/>
+    <workbookView activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>enemy_id</t>
   </si>
@@ -103,6 +103,12 @@
   </si>
   <si>
     <t>enemy_drop_value</t>
+  </si>
+  <si>
+    <t>passive_energy_value</t>
+  </si>
+  <si>
+    <t>passive_energy_interval_ms</t>
   </si>
   <si>
     <t>starting_health</t>
@@ -550,7 +556,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3204F838-D798-3BA8-BBE8-E62C7E3B17F8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E2FAAB9C-F6D8-F158-E118-D6F6CDBB7798}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -679,7 +685,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{81A3A98D-2348-6328-1256-C48FF09DB968}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8F7D31C9-D9AB-CEF8-8512-7C235552DC8F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -823,28 +829,28 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="2">
         <v>300</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="2">
         <v>20</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <v>175</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <v>10000</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <v>100</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="2">
         <v>300</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="2">
         <v>20</v>
       </c>
     </row>
@@ -861,7 +867,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CA10F698-A2B8-E168-D458-09A5F3493698}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{82AFE0DB-A6FC-AF58-73A7-417EA9ABCA6C}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -930,6 +936,22 @@
       </c>
       <c r="B8" s="2">
         <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="4">
+        <v>15000</v>
       </c>
     </row>
   </sheetData>
@@ -945,7 +967,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CF557CBB-C3F8-17D8-2DFD-001EE8494571}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{F8220421-EAA8-B1C8-1C1D-CBA99BE51538}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -962,7 +984,7 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -970,7 +992,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -978,7 +1000,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -997,7 +1019,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{36E36338-5F88-45FD-39F8-DC72C5B9A5E8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{386E72DC-F708-9472-D028-60AA684366F9}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1014,7 +1036,7 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1">
         <v>20000</v>
@@ -1022,7 +1044,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B3" s="1">
         <v>5000</v>
@@ -1030,7 +1052,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1038,7 +1060,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1046,7 +1068,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1054,7 +1076,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1062,7 +1084,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1070,7 +1092,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1078,7 +1100,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1086,7 +1108,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1094,7 +1116,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1102,7 +1124,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1110,7 +1132,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1118,7 +1140,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1126,7 +1148,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1134,7 +1156,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1142,7 +1164,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1150,7 +1172,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1158,7 +1180,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1166,7 +1188,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1174,7 +1196,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1182,7 +1204,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1190,7 +1212,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1198,7 +1220,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1206,7 +1228,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1214,7 +1236,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>

</xml_diff>

<commit_message>
added new defender the landmine
landmine take 15 to activate once placed down and explodes on contact with the enemy
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView activeTab="2"/>
+    <workbookView activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>enemy_id</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>cryogunner</t>
+  </si>
+  <si>
+    <t>landmine</t>
   </si>
   <si>
     <t>setting</t>
@@ -556,7 +559,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E2FAAB9C-F6D8-F158-E118-D6F6CDBB7798}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1D977128-4C38-EE1C-5A29-26C5CA71CEEA}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -685,7 +688,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8F7D31C9-D9AB-CEF8-8512-7C235552DC8F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{85DEED5D-1618-F9A6-D886-253399B1B618}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -854,6 +857,29 @@
         <v>20</v>
       </c>
     </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="4">
+        <v>300</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1800</v>
+      </c>
+      <c r="D7" s="4">
+        <v>25</v>
+      </c>
+      <c r="E7" s="4">
+        <v>30000</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -867,7 +893,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{82AFE0DB-A6FC-AF58-73A7-417EA9ABCA6C}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{752BC318-4ABB-7A68-71C8-72A7AD99F498}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -876,15 +902,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -892,7 +918,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -900,7 +926,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -908,7 +934,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -916,7 +942,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -924,7 +950,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -932,25 +958,25 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="4">
+      <c r="A9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="2">
         <v>25</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="4">
+      <c r="A10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="2">
         <v>15000</v>
       </c>
     </row>
@@ -967,7 +993,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{F8220421-EAA8-B1C8-1C1D-CBA99BE51538}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C9566B53-E978-158D-C4AE-4758AF23972F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -976,15 +1002,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -992,7 +1018,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1000,7 +1026,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1019,7 +1045,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{386E72DC-F708-9472-D028-60AA684366F9}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{73E0179B-571E-3DF8-04C8-226B43A69AE8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1028,15 +1054,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="1">
         <v>20000</v>
@@ -1044,7 +1070,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="1">
         <v>5000</v>
@@ -1052,7 +1078,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1060,7 +1086,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1068,7 +1094,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1076,7 +1102,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1084,7 +1110,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1092,7 +1118,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1100,7 +1126,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1108,7 +1134,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1116,7 +1142,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1124,7 +1150,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1132,7 +1158,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1140,7 +1166,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1148,7 +1174,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1156,7 +1182,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1164,7 +1190,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1172,7 +1198,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1180,7 +1206,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1188,7 +1214,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1196,7 +1222,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1204,7 +1230,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1212,7 +1238,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1220,7 +1246,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1228,7 +1254,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1236,7 +1262,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>

</xml_diff>

<commit_message>
fix generator pickups and add in more excel config gameplay settings
fixed dual barrel projectiles to use their own damage and speed settings instead of shooter values
fixed generator energy pickups remaining after the generator is destroyed or recalled
added tracking and cleanup of uncollected generator energy pickups
replaced hardcoded values with excel config settings (gen production delays, pickup values, expiration timers)
other excel config include cryo gunner slowdown values, shooter firing interval, melee enemy attack intervals, landmine arming time and blast radius,
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t>enemy_id</t>
   </si>
@@ -61,6 +61,18 @@
   </si>
   <si>
     <t>fire_interval_ms</t>
+  </si>
+  <si>
+    <t>slow_multiplier</t>
+  </si>
+  <si>
+    <t>slow_duration_ms</t>
+  </si>
+  <si>
+    <t>arming_ms</t>
+  </si>
+  <si>
+    <t>blast_radius</t>
   </si>
   <si>
     <t>shooter</t>
@@ -559,7 +571,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1D977128-4C38-EE1C-5A29-26C5CA71CEEA}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{491E9628-2964-8B48-3FA6-46B67D05051F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -688,7 +700,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{85DEED5D-1618-F9A6-D886-253399B1B618}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{179BA688-31E8-59DC-3638-71920E1D7328}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -699,6 +711,10 @@
     <col min="6" max="6" width="14.421875" customWidth="1"/>
     <col min="7" max="7" width="14.7109375" customWidth="1"/>
     <col min="8" max="8" width="16.28125" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.28125" customWidth="1"/>
+    <col min="11" max="11" width="10.00390625" customWidth="1"/>
+    <col min="12" max="12" width="10.8515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -726,10 +742,22 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
@@ -752,10 +780,22 @@
       <c r="H2" s="1">
         <v>20</v>
       </c>
+      <c r="I2" s="4">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1">
         <v>300</v>
@@ -778,10 +818,22 @@
       <c r="H3" s="1">
         <v>0</v>
       </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2">
         <v>2750</v>
@@ -804,10 +856,22 @@
       <c r="H4" s="2">
         <v>0</v>
       </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" s="2">
         <v>300</v>
@@ -828,12 +892,24 @@
         <v>300</v>
       </c>
       <c r="H5" s="2">
-        <v>20</v>
+        <v>100</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2">
         <v>300</v>
@@ -856,28 +932,55 @@
       <c r="H6" s="2">
         <v>20</v>
       </c>
+      <c r="I6" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="J6" s="4">
+        <v>1500</v>
+      </c>
+      <c r="K6" s="4">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="4">
+      <c r="A7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="2">
         <v>300</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="2">
         <v>1800</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="2">
         <v>25</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="2">
         <v>30000</v>
       </c>
-      <c r="F7" s="4">
-        <v>0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>0</v>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4">
+        <v>15000</v>
+      </c>
+      <c r="L7" s="4">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -893,7 +996,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{752BC318-4ABB-7A68-71C8-72A7AD99F498}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{34DAD346-7C33-BD28-A393-1CB2484B78F8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -902,15 +1005,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -918,7 +1021,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -926,7 +1029,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -934,7 +1037,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -942,7 +1045,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -950,7 +1053,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -958,7 +1061,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -966,7 +1069,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -974,7 +1077,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
@@ -993,7 +1096,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C9566B53-E978-158D-C4AE-4758AF23972F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{11709C38-8DC8-85D6-E905-B838C4436A98}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1002,15 +1105,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1018,7 +1121,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1026,7 +1129,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1045,7 +1148,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{73E0179B-571E-3DF8-04C8-226B43A69AE8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DD412598-3719-9674-26D2-DF158147D7C8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1054,15 +1157,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1">
         <v>20000</v>
@@ -1070,7 +1173,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B3" s="1">
         <v>5000</v>
@@ -1078,7 +1181,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1086,7 +1189,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1094,7 +1197,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1102,7 +1205,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1110,7 +1213,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1118,7 +1221,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1126,7 +1229,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1134,7 +1237,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1142,7 +1245,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1150,7 +1253,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1158,7 +1261,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1166,7 +1269,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1174,7 +1277,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1182,7 +1285,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1190,7 +1293,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1198,7 +1301,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1206,7 +1309,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1214,7 +1317,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1222,7 +1325,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1230,7 +1333,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1238,7 +1341,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1246,7 +1349,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1254,7 +1357,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1262,7 +1365,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>

</xml_diff>

<commit_message>
implement excel configd intermission between waves
added configurable intermission time between waves
implemented a cooldown displayed in the wave hud
prevent enemies from spawning during the intermission
resumes the wave after intermission is done
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView activeTab="1"/>
+    <workbookView firstSheet="1" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>enemy_id</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>level_5_wave_3_budget</t>
+  </si>
+  <si>
+    <t>wave_intermission</t>
   </si>
 </sst>
 </file>
@@ -571,7 +574,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{491E9628-2964-8B48-3FA6-46B67D05051F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6A5DE0E8-AD98-609C-38B4-9750F646FE28}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -700,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{179BA688-31E8-59DC-3638-71920E1D7328}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{44BAFB0B-0228-5E9E-7738-C07E0D752727}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -996,7 +999,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{34DAD346-7C33-BD28-A393-1CB2484B78F8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{23E6A34F-6088-DB95-AAA2-B93AEF64B938}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1096,7 +1099,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{11709C38-8DC8-85D6-E905-B838C4436A98}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{2BF2C2E8-10FF-0A84-D2B8-AA15A0F7D913}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1148,7 +1151,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DD412598-3719-9674-26D2-DF158147D7C8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0DA61758-EE38-1E88-6F51-02AD5FCFF2D8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1369,6 +1372,14 @@
       </c>
       <c r="B27" s="2">
         <v>110</v>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B28" s="4">
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
integrate overlord boss encounter into level 5
added a final boss encounter after level 5, wave 3
integrated the overworld into the existing gameplay and collision systems
implemented basic boss projectile attacks across multiple ;lanes
fixed an issue where not all5 lanes would shoot the boss
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView/>
+    <workbookView firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -272,13 +272,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -577,7 +576,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5C2647B8-36F5-FEE8-8A08-E4198F463FF9}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{43CCF585-D3AA-C538-E238-CBF172DCE51A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -694,28 +693,28 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>15000</v>
       </c>
-      <c r="C5" s="3">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3">
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
         <v>200</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>2000</v>
       </c>
-      <c r="F5" s="3">
-        <v>0</v>
-      </c>
-      <c r="G5" s="3">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3">
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -732,7 +731,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{56B12F13-E475-FA58-C088-3EB410068C78}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E91C53C8-57C8-4BCA-E488-891638DCA8A2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -759,7 +758,7 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -804,7 +803,7 @@
         <v>7500</v>
       </c>
       <c r="F2" s="1">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1">
         <v>300</v>
@@ -918,7 +917,7 @@
         <v>12000</v>
       </c>
       <c r="F5" s="2">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="G5" s="2">
         <v>300</v>
@@ -956,7 +955,7 @@
         <v>10000</v>
       </c>
       <c r="F6" s="2">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="G6" s="2">
         <v>300</v>
@@ -1028,7 +1027,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5468AFA7-2128-DA0A-B2C8-E435A468B718}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{340DF0F8-0E8B-7E9F-B308-DDADF1AF6BCB}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1048,7 +1047,7 @@
         <v>28</v>
       </c>
       <c r="B2" s="1">
-        <v>500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
@@ -1128,7 +1127,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{08B97A0A-4781-8DE2-B125-FFE620B49D3D}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{53978668-9AB8-4C35-7468-7501EDA94626}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1180,7 +1179,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3E80E868-9FD8-1F68-70D5-39CD48CD5448}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{41BEB57D-50D8-4B08-B6A8-209BC3D13E48}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1200,7 +1199,7 @@
         <v>40</v>
       </c>
       <c r="B2" s="1">
-        <v>20000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
@@ -1208,7 +1207,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="1">
-        <v>5000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">

</xml_diff>

<commit_message>
remove all the lint warnings
lint warnings removed
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -576,7 +576,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{43CCF585-D3AA-C538-E238-CBF172DCE51A}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5943C3D2-BE58-95CD-0D28-E21113C3C194}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -731,7 +731,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E91C53C8-57C8-4BCA-E488-891638DCA8A2}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0FEA50C8-9559-A369-22D6-1261BCA443D1}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1027,7 +1027,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{340DF0F8-0E8B-7E9F-B308-DDADF1AF6BCB}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D804E55E-7E98-3A48-5154-5931A463F7C8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1127,7 +1127,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{53978668-9AB8-4C35-7468-7501EDA94626}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E200CFF8-C071-D8FD-ED41-9281A27DAB98}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1179,7 +1179,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{41BEB57D-50D8-4B08-B6A8-209BC3D13E48}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4F99B268-DD8B-B518-3481-2A5BB56931B8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>

</xml_diff>

<commit_message>
added new enemy drone enemy
the drone enemy flyies over every defender but it can still be destroyed by the shooters
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView firstSheet="1" activeTab="2"/>
+    <workbookView/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>enemy_id</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>boss</t>
+  </si>
+  <si>
+    <t>drone</t>
   </si>
   <si>
     <t>defender_id</t>
@@ -272,12 +275,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -576,7 +580,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5943C3D2-BE58-95CD-0D28-E21113C3C194}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1EB2C8F8-0641-4DD8-B244-4C7E988AD928}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -718,6 +722,32 @@
         <v>0</v>
       </c>
     </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="3">
+        <v>300</v>
+      </c>
+      <c r="C6" s="3">
+        <v>18</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -731,7 +761,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0FEA50C8-9559-A369-22D6-1261BCA443D1}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{423CBF58-AE68-4838-6E28-D41670AC8028}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -750,7 +780,7 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -758,14 +788,14 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>13</v>
+      <c r="D1" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -774,21 +804,21 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
@@ -826,7 +856,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1">
         <v>300</v>
@@ -864,7 +894,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" s="2">
         <v>2750</v>
@@ -902,7 +932,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2">
         <v>300</v>
@@ -940,7 +970,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2">
         <v>300</v>
@@ -978,7 +1008,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" s="2">
         <v>300</v>
@@ -1027,7 +1057,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D804E55E-7E98-3A48-5154-5931A463F7C8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B1A27251-AE08-EFB4-14D8-E42DFB4BC443}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1036,15 +1066,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1052,7 +1082,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1060,7 +1090,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1068,7 +1098,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1076,7 +1106,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1084,7 +1114,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1092,7 +1122,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1100,7 +1130,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1108,7 +1138,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
@@ -1127,7 +1157,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E200CFF8-C071-D8FD-ED41-9281A27DAB98}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FDF2A2C3-3E36-BB14-2B38-96EDD13288D8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1136,15 +1166,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1152,7 +1182,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1160,7 +1190,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1179,7 +1209,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4F99B268-DD8B-B518-3481-2A5BB56931B8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{94918448-FE48-2E4B-61D7-C309BF2F9FDA}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1188,15 +1218,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1">
         <v>1000</v>
@@ -1204,7 +1234,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1212,7 +1242,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1220,7 +1250,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1228,7 +1258,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1236,7 +1266,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1244,7 +1274,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1252,7 +1282,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1260,7 +1290,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1268,7 +1298,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1276,7 +1306,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1284,7 +1314,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1292,7 +1322,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1300,7 +1330,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1308,7 +1338,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1316,7 +1346,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1324,7 +1354,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1332,7 +1362,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1340,7 +1370,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1348,7 +1378,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1356,7 +1386,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1364,7 +1394,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1372,7 +1402,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1380,7 +1410,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1388,7 +1418,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1396,7 +1426,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>
@@ -1404,7 +1434,7 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B28" s="2">
         <v>10000</v>

</xml_diff>

<commit_message>
added new enemy hijacker
the hijacker enemy falls from above and steals one of your defenders
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>enemy_id</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>drone</t>
+  </si>
+  <si>
+    <t>hijacker</t>
   </si>
   <si>
     <t>defender_id</t>
@@ -580,7 +583,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1EB2C8F8-0641-4DD8-B244-4C7E988AD928}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4F2851D3-51E8-DCAB-FD88-426847D8DADC}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -723,28 +726,54 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>300</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>18</v>
       </c>
-      <c r="D6" s="3">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>0</v>
-      </c>
-      <c r="F6" s="3">
-        <v>0</v>
-      </c>
-      <c r="G6" s="3">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3">
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3">
+        <v>450</v>
+      </c>
+      <c r="C7" s="3">
+        <v>40</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
         <v>0</v>
       </c>
     </row>
@@ -761,7 +790,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{423CBF58-AE68-4838-6E28-D41670AC8028}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{30985298-EFE8-3288-D738-A9E379D30B78}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -780,7 +809,7 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -789,13 +818,13 @@
         <v>3</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -804,21 +833,21 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
@@ -856,7 +885,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1">
         <v>300</v>
@@ -894,7 +923,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2">
         <v>2750</v>
@@ -932,7 +961,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2">
         <v>300</v>
@@ -970,7 +999,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2">
         <v>300</v>
@@ -1008,7 +1037,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2">
         <v>300</v>
@@ -1057,7 +1086,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B1A27251-AE08-EFB4-14D8-E42DFB4BC443}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8809DB18-D06E-4768-9B7E-288175D5ABD2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1066,15 +1095,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1082,7 +1111,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1090,7 +1119,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1098,7 +1127,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1106,7 +1135,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1114,7 +1143,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1122,7 +1151,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1130,7 +1159,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1138,7 +1167,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
@@ -1157,7 +1186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FDF2A2C3-3E36-BB14-2B38-96EDD13288D8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{2312CD68-2558-3048-D71C-FCA891CCBFA8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1166,15 +1195,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1182,7 +1211,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1190,7 +1219,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1209,7 +1238,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{94918448-FE48-2E4B-61D7-C309BF2F9FDA}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{720142E8-424E-B244-2D3F-D209249D5C38}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1218,15 +1247,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" s="1">
         <v>1000</v>
@@ -1234,7 +1263,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1242,7 +1271,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1250,7 +1279,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1258,7 +1287,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1266,7 +1295,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1274,7 +1303,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1282,7 +1311,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1290,7 +1319,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1298,7 +1327,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1306,7 +1335,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1314,7 +1343,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1322,7 +1351,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1330,7 +1359,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1338,7 +1367,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1346,7 +1375,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1354,7 +1383,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1362,7 +1391,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1370,7 +1399,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1378,7 +1407,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1386,7 +1415,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1394,7 +1423,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1402,7 +1431,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1410,7 +1439,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1418,7 +1447,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1426,7 +1455,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>
@@ -1434,7 +1463,7 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B28" s="2">
         <v>10000</v>

</xml_diff>

<commit_message>
Add defender specific upgrade costs using the spreadsheet
Added individual upgrade costs for each defender using the Excel spreadsheet
Upgrading now checks and deducts energy, updates the HUD, and prevents upgrades when energy is insufficient.
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView activeTab="4"/>
+    <workbookView activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>enemy_id</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>blast_radius</t>
+  </si>
+  <si>
+    <t>upgrade_cost</t>
   </si>
   <si>
     <t>shooter</t>
@@ -278,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -287,6 +290,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -582,7 +586,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1B53BF6A-C134-5EF5-0628-B066F19B005E}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{93C95D98-AD88-01CC-0968-883B09157897}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -789,7 +793,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B42F2728-3176-3228-0AED-0A84B72AF307}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A5A47708-5A08-F328-7D45-7382B44A230E}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -843,10 +847,13 @@
       <c r="L1" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="M1" s="4" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
@@ -881,10 +888,13 @@
       <c r="L2" s="2">
         <v>0</v>
       </c>
+      <c r="M2" s="4">
+        <v>100</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1">
         <v>300</v>
@@ -919,10 +929,13 @@
       <c r="L3" s="2">
         <v>0</v>
       </c>
+      <c r="M3" s="4">
+        <v>75</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="2">
         <v>2750</v>
@@ -957,10 +970,13 @@
       <c r="L4" s="2">
         <v>0</v>
       </c>
+      <c r="M4" s="4">
+        <v>75</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="2">
         <v>300</v>
@@ -995,10 +1011,13 @@
       <c r="L5" s="2">
         <v>0</v>
       </c>
+      <c r="M5" s="4">
+        <v>150</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="2">
         <v>300</v>
@@ -1033,10 +1052,13 @@
       <c r="L6" s="2">
         <v>0</v>
       </c>
+      <c r="M6" s="4">
+        <v>120</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" s="2">
         <v>300</v>
@@ -1071,6 +1093,12 @@
       <c r="L7" s="2">
         <v>90</v>
       </c>
+      <c r="M7" s="4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="4"/>
     </row>
   </sheetData>
   <printOptions/>
@@ -1085,7 +1113,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{84669322-99EC-B2B8-B933-6DB5D6A39C68}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E099C278-B47F-9398-8F9C-A27AB8F654EB}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1094,15 +1122,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1110,7 +1138,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1118,7 +1146,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1126,7 +1154,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1134,7 +1162,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1142,7 +1170,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1150,7 +1178,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1158,7 +1186,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1166,7 +1194,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
@@ -1185,7 +1213,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B9442BF8-A958-1508-BB65-9B4C2DCAABB8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4838F7C9-E958-7003-46C4-BA024B9A97A8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1194,15 +1222,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1210,7 +1238,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1218,7 +1246,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1237,7 +1265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{F549372F-1565-4548-A208-6A3C3D82DE71}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{02923698-6B86-5F6D-D4E8-BF186D77779F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1246,15 +1274,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1">
         <v>1000</v>
@@ -1262,7 +1290,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1270,7 +1298,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1278,7 +1306,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1286,7 +1314,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1294,7 +1322,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1302,7 +1330,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1310,7 +1338,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1318,7 +1346,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1326,7 +1354,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1334,7 +1362,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1342,7 +1370,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1350,7 +1378,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1358,7 +1386,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1366,7 +1394,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1374,7 +1402,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1382,7 +1410,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1390,7 +1418,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1398,7 +1426,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1406,7 +1434,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1414,7 +1442,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1422,7 +1450,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1430,7 +1458,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1438,7 +1466,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1446,7 +1474,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1454,7 +1482,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>
@@ -1462,7 +1490,7 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B28" s="2">
         <v>10000</v>

</xml_diff>

<commit_message>
implement level-based defender unlock system and locked toolbar indicators
implemented level based defender unlocking across the five levels
added unlock requirements for each defender type
prevented locked defenders from being selected, dragged or placed
added greyed out toolbar icons with LOCKED labels and required unlock levels
updated the toolbar so it can automatically unlock defenders when progressing to the required level
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -281,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -290,7 +290,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -586,7 +585,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{93C95D98-AD88-01CC-0968-883B09157897}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1147A3AD-A958-4DAC-0DD7-CAC214F30468}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -793,7 +792,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A5A47708-5A08-F328-7D45-7382B44A230E}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6F8926B8-4C68-C768-11A8-1679482114D8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -847,7 +846,7 @@
       <c r="L1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -888,7 +887,7 @@
       <c r="L2" s="2">
         <v>0</v>
       </c>
-      <c r="M2" s="4">
+      <c r="M2" s="2">
         <v>100</v>
       </c>
     </row>
@@ -929,7 +928,7 @@
       <c r="L3" s="2">
         <v>0</v>
       </c>
-      <c r="M3" s="4">
+      <c r="M3" s="2">
         <v>75</v>
       </c>
     </row>
@@ -970,7 +969,7 @@
       <c r="L4" s="2">
         <v>0</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="2">
         <v>75</v>
       </c>
     </row>
@@ -1011,7 +1010,7 @@
       <c r="L5" s="2">
         <v>0</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="2">
         <v>150</v>
       </c>
     </row>
@@ -1052,7 +1051,7 @@
       <c r="L6" s="2">
         <v>0</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="2">
         <v>120</v>
       </c>
     </row>
@@ -1093,12 +1092,12 @@
       <c r="L7" s="2">
         <v>90</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="2">
         <v>50</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="4"/>
+      <c r="A8" s="2"/>
     </row>
   </sheetData>
   <printOptions/>
@@ -1113,7 +1112,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E099C278-B47F-9398-8F9C-A27AB8F654EB}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CAF0EED8-6FA8-09A8-0E11-F7C24D55CBE8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1213,7 +1212,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4838F7C9-E958-7003-46C4-BA024B9A97A8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0DDB8588-6C93-4428-A4A8-D9242F385AEC}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1265,7 +1264,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{02923698-6B86-5F6D-D4E8-BF186D77779F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5B0E9E48-36D1-148F-28DE-57E2990B5A85}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>

</xml_diff>

<commit_message>
Implemented Level 2 Shooter damage upgrade
Added upgrade damage multipliers to Excel configuration
Exported upgrade multipliers to CSV
Implemented 1.5x projectile damage increase for Level 2 Shooter
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t>enemy_id</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>upgrade_cost</t>
+  </si>
+  <si>
+    <t>upgrade_damage_multiplier</t>
   </si>
   <si>
     <t>shooter</t>
@@ -281,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -290,6 +293,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,7 +589,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1147A3AD-A958-4DAC-0DD7-CAC214F30468}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{07BFA448-13F8-6B15-8878-658BBBDFE92A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -792,7 +796,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6F8926B8-4C68-C768-11A8-1679482114D8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{722AE02E-71E9-1348-8AC8-A1C2778C0A38}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -849,10 +853,13 @@
       <c r="M1" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="N1" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
@@ -890,10 +897,13 @@
       <c r="M2" s="2">
         <v>100</v>
       </c>
+      <c r="N2" s="4">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1">
         <v>300</v>
@@ -931,10 +941,13 @@
       <c r="M3" s="2">
         <v>75</v>
       </c>
+      <c r="N3" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="2">
         <v>2750</v>
@@ -972,10 +985,13 @@
       <c r="M4" s="2">
         <v>75</v>
       </c>
+      <c r="N4" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2">
         <v>300</v>
@@ -1013,10 +1029,13 @@
       <c r="M5" s="2">
         <v>150</v>
       </c>
+      <c r="N5" s="4">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2">
         <v>300</v>
@@ -1054,10 +1073,13 @@
       <c r="M6" s="2">
         <v>120</v>
       </c>
+      <c r="N6" s="4">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B7" s="2">
         <v>300</v>
@@ -1094,6 +1116,9 @@
       </c>
       <c r="M7" s="2">
         <v>50</v>
+      </c>
+      <c r="N7" s="4">
+        <v>1.5</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -1112,7 +1137,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CAF0EED8-6FA8-09A8-0E11-F7C24D55CBE8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1775B853-9AC8-B1E8-3A98-B21D21FC4159}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1121,15 +1146,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1137,7 +1162,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1145,7 +1170,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1153,7 +1178,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1161,7 +1186,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1169,7 +1194,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1177,7 +1202,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1185,7 +1210,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1193,7 +1218,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
@@ -1212,7 +1237,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0DDB8588-6C93-4428-A4A8-D9242F385AEC}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5A0DCFD8-2838-A908-7F7C-E2C8E2638A4E}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1221,15 +1246,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1237,7 +1262,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1245,7 +1270,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1264,7 +1289,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5B0E9E48-36D1-148F-28DE-57E2990B5A85}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FC346EE5-AFB3-ED28-0428-ED9F1D07BB18}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1273,15 +1298,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1">
         <v>1000</v>
@@ -1289,7 +1314,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1297,7 +1322,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1305,7 +1330,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1313,7 +1338,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1321,7 +1346,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1329,7 +1354,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1337,7 +1362,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1345,7 +1370,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1353,7 +1378,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1361,7 +1386,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1369,7 +1394,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1377,7 +1402,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1385,7 +1410,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1393,7 +1418,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1401,7 +1426,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1409,7 +1434,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1417,7 +1442,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1425,7 +1450,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1433,7 +1458,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1441,7 +1466,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1449,7 +1474,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1457,7 +1482,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1465,7 +1490,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1473,7 +1498,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1481,7 +1506,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>
@@ -1489,7 +1514,7 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B28" s="2">
         <v>10000</v>

</xml_diff>

<commit_message>
Added Level 2 upgrades for Generator and Barricade
Generator produces 1.5x more energy when upgraded
Barricade gains 1.5x more health at Level 2
Upgrade health and energy multipliers are now used in the spreadsheet too so easy to change
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>enemy_id</t>
   </si>
@@ -88,6 +88,12 @@
   </si>
   <si>
     <t>upgrade_damage_multiplier</t>
+  </si>
+  <si>
+    <t>upgrade_energy_multiplier</t>
+  </si>
+  <si>
+    <t>upgrade_health_multiplier</t>
   </si>
   <si>
     <t>shooter</t>
@@ -589,7 +595,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{07BFA448-13F8-6B15-8878-658BBBDFE92A}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6369BAFB-C458-6793-8D08-4960C235F276}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -796,7 +802,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{722AE02E-71E9-1348-8AC8-A1C2778C0A38}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{327F2108-8708-F168-DA58-0866033646B8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -856,10 +862,16 @@
       <c r="N1" s="4" t="s">
         <v>23</v>
       </c>
+      <c r="O1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
@@ -900,10 +912,16 @@
       <c r="N2" s="4">
         <v>1.5</v>
       </c>
+      <c r="O2" s="4">
+        <v>1</v>
+      </c>
+      <c r="P2" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B3" s="1">
         <v>300</v>
@@ -944,10 +962,16 @@
       <c r="N3" s="4">
         <v>1</v>
       </c>
+      <c r="O3" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="P3" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2">
         <v>2750</v>
@@ -988,10 +1012,16 @@
       <c r="N4" s="4">
         <v>1</v>
       </c>
+      <c r="O4" s="4">
+        <v>1</v>
+      </c>
+      <c r="P4" s="4">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="2">
         <v>300</v>
@@ -1032,10 +1062,16 @@
       <c r="N5" s="4">
         <v>1.5</v>
       </c>
+      <c r="O5" s="4">
+        <v>1</v>
+      </c>
+      <c r="P5" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B6" s="2">
         <v>300</v>
@@ -1076,10 +1112,16 @@
       <c r="N6" s="4">
         <v>1.5</v>
       </c>
+      <c r="O6" s="4">
+        <v>1</v>
+      </c>
+      <c r="P6" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7" s="2">
         <v>300</v>
@@ -1119,6 +1161,12 @@
       </c>
       <c r="N7" s="4">
         <v>1.5</v>
+      </c>
+      <c r="O7" s="4">
+        <v>1</v>
+      </c>
+      <c r="P7" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -1137,7 +1185,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1775B853-9AC8-B1E8-3A98-B21D21FC4159}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C5AE0CE8-6793-710E-020F-2DAB0F060B08}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1146,15 +1194,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1162,7 +1210,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1170,7 +1218,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1178,7 +1226,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1186,7 +1234,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1194,7 +1242,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1202,7 +1250,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1210,7 +1258,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1218,7 +1266,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
@@ -1237,7 +1285,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5A0DCFD8-2838-A908-7F7C-E2C8E2638A4E}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B2417348-F922-5338-1CC8-3E62D799F0F8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1246,15 +1294,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1262,7 +1310,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1270,7 +1318,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1289,7 +1337,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FC346EE5-AFB3-ED28-0428-ED9F1D07BB18}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{02819889-2FD8-F6BB-87B8-BA69741B3C5D}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1298,15 +1346,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1">
         <v>1000</v>
@@ -1314,7 +1362,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1322,7 +1370,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B4" s="1">
         <v>0.6</v>
@@ -1330,7 +1378,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" s="1">
         <v>0.3</v>
@@ -1338,7 +1386,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -1346,7 +1394,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
@@ -1354,7 +1402,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B8" s="2">
         <v>3</v>
@@ -1362,7 +1410,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -1370,7 +1418,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1378,7 +1426,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B11" s="2">
         <v>3</v>
@@ -1386,7 +1434,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1394,7 +1442,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1402,7 +1450,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B14" s="2">
         <v>10</v>
@@ -1410,7 +1458,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B15" s="2">
         <v>20</v>
@@ -1418,7 +1466,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B16" s="2">
         <v>15</v>
@@ -1426,7 +1474,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B17" s="2">
         <v>20</v>
@@ -1434,7 +1482,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B18" s="2">
         <v>30</v>
@@ -1442,7 +1490,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B19" s="2">
         <v>40</v>
@@ -1450,7 +1498,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B20" s="2">
         <v>50</v>
@@ -1458,7 +1506,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B21" s="2">
         <v>60</v>
@@ -1466,7 +1514,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B22" s="2">
         <v>50</v>
@@ -1474,7 +1522,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B23" s="2">
         <v>65</v>
@@ -1482,7 +1530,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B24" s="2">
         <v>80</v>
@@ -1490,7 +1538,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B25" s="2">
         <v>70</v>
@@ -1498,7 +1546,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B26" s="2">
         <v>90</v>
@@ -1506,7 +1554,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B27" s="2">
         <v>110</v>
@@ -1514,7 +1562,7 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B28" s="2">
         <v>10000</v>

</xml_diff>

<commit_message>
integrate new enemy types (hijacker and drone) into waves and implement level-based difficulty scaling (increase)
integrated droneenemy and hijackernemy into the wave spawning system
added configurable spawn probabilities and wave costs for both new enemies
connected hijacker movement, defender targeting, stealing and escape behaviour
implemented increasing enemy health and damage across all five levels
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView activeTab="1"/>
+    <workbookView activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
     <t>enemy_id</t>
   </si>
@@ -114,6 +114,9 @@
     <t>landmine</t>
   </si>
   <si>
+    <t>.</t>
+  </si>
+  <si>
     <t>setting</t>
   </si>
   <si>
@@ -168,6 +171,12 @@
     <t>ranged_spawn_probability</t>
   </si>
   <si>
+    <t>hijacker_spawn_probability</t>
+  </si>
+  <si>
+    <t>drone_spawn_probability</t>
+  </si>
+  <si>
     <t>crusher_spawn_probability</t>
   </si>
   <si>
@@ -195,6 +204,12 @@
     <t>ranged_wave_cost</t>
   </si>
   <si>
+    <t>hijacker_wave_cost</t>
+  </si>
+  <si>
+    <t>drone_wave_cost</t>
+  </si>
+  <si>
     <t>crusher_wave_cost</t>
   </si>
   <si>
@@ -235,6 +250,12 @@
   </si>
   <si>
     <t>wave_intermission</t>
+  </si>
+  <si>
+    <t>enemy_health_increase_per_level</t>
+  </si>
+  <si>
+    <t>enemy_damage_increase_per_level</t>
   </si>
 </sst>
 </file>
@@ -290,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -299,6 +320,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -595,7 +617,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6369BAFB-C458-6793-8D08-4960C235F276}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{17B26627-4658-1E69-E178-79CD8F678468}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -802,7 +824,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{327F2108-8708-F168-DA58-0866033646B8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3A4775A7-619D-FD08-96FE-A3BF007A5057}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -817,6 +839,10 @@
     <col min="10" max="10" width="16.28125" customWidth="1"/>
     <col min="11" max="11" width="10.00390625" customWidth="1"/>
     <col min="12" max="12" width="10.8515625" customWidth="1"/>
+    <col min="13" max="13" width="12.00390625" customWidth="1"/>
+    <col min="14" max="14" width="24.7109375" customWidth="1"/>
+    <col min="15" max="15" width="23.7109375" customWidth="1"/>
+    <col min="16" max="16" width="23.28125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -859,13 +885,13 @@
       <c r="M1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -909,13 +935,13 @@
       <c r="M2" s="2">
         <v>100</v>
       </c>
-      <c r="N2" s="4">
+      <c r="N2" s="2">
         <v>1.5</v>
       </c>
-      <c r="O2" s="4">
+      <c r="O2" s="2">
         <v>1</v>
       </c>
-      <c r="P2" s="4">
+      <c r="P2" s="2">
         <v>1</v>
       </c>
     </row>
@@ -959,13 +985,13 @@
       <c r="M3" s="2">
         <v>75</v>
       </c>
-      <c r="N3" s="4">
+      <c r="N3" s="2">
         <v>1</v>
       </c>
-      <c r="O3" s="4">
+      <c r="O3" s="2">
         <v>1.5</v>
       </c>
-      <c r="P3" s="4">
+      <c r="P3" s="2">
         <v>1</v>
       </c>
     </row>
@@ -1009,13 +1035,13 @@
       <c r="M4" s="2">
         <v>75</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="2">
         <v>1</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="2">
         <v>1</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="2">
         <v>1.5</v>
       </c>
     </row>
@@ -1059,13 +1085,13 @@
       <c r="M5" s="2">
         <v>150</v>
       </c>
-      <c r="N5" s="4">
+      <c r="N5" s="2">
         <v>1.5</v>
       </c>
-      <c r="O5" s="4">
+      <c r="O5" s="2">
         <v>1</v>
       </c>
-      <c r="P5" s="4">
+      <c r="P5" s="2">
         <v>1</v>
       </c>
     </row>
@@ -1109,13 +1135,13 @@
       <c r="M6" s="2">
         <v>120</v>
       </c>
-      <c r="N6" s="4">
+      <c r="N6" s="2">
         <v>1.5</v>
       </c>
-      <c r="O6" s="4">
+      <c r="O6" s="2">
         <v>1</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="2">
         <v>1</v>
       </c>
     </row>
@@ -1159,18 +1185,23 @@
       <c r="M7" s="2">
         <v>50</v>
       </c>
-      <c r="N7" s="4">
+      <c r="N7" s="2">
         <v>1.5</v>
       </c>
-      <c r="O7" s="4">
+      <c r="O7" s="2">
         <v>1</v>
       </c>
-      <c r="P7" s="4">
+      <c r="P7" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2"/>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="M18" s="4" t="s">
+        <v>32</v>
+      </c>
     </row>
   </sheetData>
   <printOptions/>
@@ -1185,7 +1216,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C5AE0CE8-6793-710E-020F-2DAB0F060B08}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9A67F351-5B48-7EB4-C418-995218B62B61}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1194,15 +1225,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1210,7 +1241,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1218,7 +1249,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1226,7 +1257,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1234,7 +1265,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1242,7 +1273,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1250,7 +1281,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1258,7 +1289,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1266,7 +1297,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
@@ -1285,7 +1316,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B2417348-F922-5338-1CC8-3E62D799F0F8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{541411E8-C1A8-1FB8-09D8-0ED3EA313A87}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1294,15 +1325,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1310,7 +1341,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1318,7 +1349,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1337,24 +1368,24 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{02819889-2FD8-F6BB-87B8-BA69741B3C5D}" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:T200"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B7220D78-D478-C2BF-79C8-39C007D22C68}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T204"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="24.57421875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" s="1">
         <v>1000</v>
@@ -1362,7 +1393,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1370,203 +1401,1128 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" s="1">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" s="1">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="2">
-        <v>0.1</v>
+      <c r="A6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0.15</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="2">
-        <v>1</v>
-      </c>
+      <c r="A7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="C7" s="5"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B8" s="2">
-        <v>3</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="C8" s="5"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B9" s="2">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C9" s="5"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
       </c>
+      <c r="C10" s="5"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B11" s="2">
-        <v>3</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
       </c>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="2">
-        <v>5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B14" s="2">
-        <v>10</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="2">
-        <v>20</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C15" s="5"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B16" s="2">
+        <v>10</v>
+      </c>
+      <c r="C16" s="5"/>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="4">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="2">
-        <v>20</v>
-      </c>
+      <c r="C17" s="5"/>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="2">
-        <v>30</v>
-      </c>
+      <c r="A18" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="4">
+        <v>10</v>
+      </c>
+      <c r="C18" s="5"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B19" s="2">
-        <v>40</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="C19" s="5"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B20" s="2">
-        <v>50</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="C20" s="5"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B21" s="2">
-        <v>60</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="C21" s="5"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B22" s="2">
-        <v>50</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="C22" s="5"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B23" s="2">
-        <v>65</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C23" s="5"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B24" s="2">
-        <v>80</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="C24" s="5"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B25" s="2">
-        <v>70</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="C25" s="5"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B26" s="2">
-        <v>90</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="C26" s="5"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B27" s="2">
-        <v>110</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="C27" s="5"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B28" s="2">
+        <v>80</v>
+      </c>
+      <c r="C28" s="5"/>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" s="2">
+        <v>70</v>
+      </c>
+      <c r="C29" s="5"/>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B30" s="2">
+        <v>90</v>
+      </c>
+      <c r="C30" s="5"/>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" s="2">
+        <v>110</v>
+      </c>
+      <c r="C31" s="5"/>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" s="2">
         <v>10000</v>
       </c>
+      <c r="C32" s="5"/>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="C33" s="5"/>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="C34" s="5"/>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="5"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="5"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+    </row>
+    <row r="41" ht="15" customHeight="1">
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+    </row>
+    <row r="42" ht="15" customHeight="1">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+    </row>
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="5"/>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5"/>
+    </row>
+    <row r="45" ht="15" customHeight="1">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
+    </row>
+    <row r="47" ht="15" customHeight="1">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+    </row>
+    <row r="49" ht="15" customHeight="1">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+    </row>
+    <row r="50" ht="15" customHeight="1">
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
+      <c r="C50" s="5"/>
+    </row>
+    <row r="51" ht="15" customHeight="1">
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="5"/>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" s="5"/>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5"/>
+    </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="A54" s="5"/>
+      <c r="B54" s="5"/>
+      <c r="C54" s="5"/>
+    </row>
+    <row r="55" ht="15" customHeight="1">
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
+    </row>
+    <row r="56" ht="15" customHeight="1">
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+    </row>
+    <row r="57" ht="15" customHeight="1">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
+    </row>
+    <row r="58" ht="15" customHeight="1">
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
+    </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+    </row>
+    <row r="60" ht="15" customHeight="1">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="5"/>
+    </row>
+    <row r="61" ht="15" customHeight="1">
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="A62" s="5"/>
+      <c r="B62" s="5"/>
+      <c r="C62" s="5"/>
+    </row>
+    <row r="63" ht="15" customHeight="1">
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
+    </row>
+    <row r="64" ht="15" customHeight="1">
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
+      <c r="C64" s="5"/>
+    </row>
+    <row r="65" ht="15" customHeight="1">
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
+      <c r="C65" s="5"/>
+    </row>
+    <row r="66" ht="15" customHeight="1">
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
+      <c r="C66" s="5"/>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="A67" s="5"/>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+    </row>
+    <row r="68" ht="15" customHeight="1">
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+    </row>
+    <row r="69" ht="15" customHeight="1">
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+    </row>
+    <row r="70" ht="15" customHeight="1">
+      <c r="A70" s="5"/>
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
+    </row>
+    <row r="71" ht="15" customHeight="1">
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
+      <c r="C71" s="5"/>
+    </row>
+    <row r="72" ht="15" customHeight="1">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5"/>
+      <c r="C72" s="5"/>
+    </row>
+    <row r="73" ht="15" customHeight="1">
+      <c r="A73" s="5"/>
+      <c r="B73" s="5"/>
+      <c r="C73" s="5"/>
+    </row>
+    <row r="74" ht="15" customHeight="1">
+      <c r="A74" s="5"/>
+      <c r="B74" s="5"/>
+      <c r="C74" s="5"/>
+    </row>
+    <row r="75" ht="15" customHeight="1">
+      <c r="A75" s="5"/>
+      <c r="B75" s="5"/>
+      <c r="C75" s="5"/>
+    </row>
+    <row r="76" ht="15" customHeight="1">
+      <c r="A76" s="5"/>
+      <c r="B76" s="5"/>
+      <c r="C76" s="5"/>
+    </row>
+    <row r="77" ht="15" customHeight="1">
+      <c r="A77" s="5"/>
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+    </row>
+    <row r="78" ht="15" customHeight="1">
+      <c r="A78" s="5"/>
+      <c r="B78" s="5"/>
+      <c r="C78" s="5"/>
+    </row>
+    <row r="79" ht="15" customHeight="1">
+      <c r="A79" s="5"/>
+      <c r="B79" s="5"/>
+      <c r="C79" s="5"/>
+    </row>
+    <row r="80" ht="15" customHeight="1">
+      <c r="A80" s="5"/>
+      <c r="B80" s="5"/>
+      <c r="C80" s="5"/>
+    </row>
+    <row r="81" ht="15" customHeight="1">
+      <c r="A81" s="5"/>
+      <c r="B81" s="5"/>
+      <c r="C81" s="5"/>
+    </row>
+    <row r="82" ht="15" customHeight="1">
+      <c r="A82" s="5"/>
+      <c r="B82" s="5"/>
+      <c r="C82" s="5"/>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="5"/>
+      <c r="B83" s="5"/>
+      <c r="C83" s="5"/>
+    </row>
+    <row r="84" ht="15" customHeight="1">
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
+      <c r="C84" s="5"/>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
+      <c r="C85" s="5"/>
+    </row>
+    <row r="86" ht="15" customHeight="1">
+      <c r="A86" s="5"/>
+      <c r="B86" s="5"/>
+      <c r="C86" s="5"/>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" s="5"/>
+      <c r="B87" s="5"/>
+      <c r="C87" s="5"/>
+    </row>
+    <row r="88" ht="15" customHeight="1">
+      <c r="A88" s="5"/>
+      <c r="B88" s="5"/>
+      <c r="C88" s="5"/>
+    </row>
+    <row r="89" ht="15" customHeight="1">
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
+      <c r="C89" s="5"/>
+    </row>
+    <row r="90" ht="15" customHeight="1">
+      <c r="A90" s="5"/>
+      <c r="B90" s="5"/>
+      <c r="C90" s="5"/>
+    </row>
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="5"/>
+      <c r="B91" s="5"/>
+      <c r="C91" s="5"/>
+    </row>
+    <row r="92" ht="15" customHeight="1">
+      <c r="A92" s="5"/>
+      <c r="B92" s="5"/>
+      <c r="C92" s="5"/>
+    </row>
+    <row r="93" ht="15" customHeight="1">
+      <c r="A93" s="5"/>
+      <c r="B93" s="5"/>
+      <c r="C93" s="5"/>
+    </row>
+    <row r="94" ht="15" customHeight="1">
+      <c r="A94" s="5"/>
+      <c r="B94" s="5"/>
+      <c r="C94" s="5"/>
+    </row>
+    <row r="95" ht="15" customHeight="1">
+      <c r="A95" s="5"/>
+      <c r="B95" s="5"/>
+      <c r="C95" s="5"/>
+    </row>
+    <row r="96" ht="15" customHeight="1">
+      <c r="A96" s="5"/>
+      <c r="B96" s="5"/>
+      <c r="C96" s="5"/>
+    </row>
+    <row r="97" ht="15" customHeight="1">
+      <c r="A97" s="5"/>
+      <c r="B97" s="5"/>
+      <c r="C97" s="5"/>
+    </row>
+    <row r="98" ht="15" customHeight="1">
+      <c r="A98" s="5"/>
+      <c r="B98" s="5"/>
+      <c r="C98" s="5"/>
+    </row>
+    <row r="99" ht="15" customHeight="1">
+      <c r="A99" s="5"/>
+      <c r="B99" s="5"/>
+      <c r="C99" s="5"/>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="5"/>
+      <c r="B100" s="5"/>
+      <c r="C100" s="5"/>
+    </row>
+    <row r="101" ht="15" customHeight="1">
+      <c r="A101" s="5"/>
+      <c r="B101" s="5"/>
+      <c r="C101" s="5"/>
+    </row>
+    <row r="102" ht="15" customHeight="1">
+      <c r="A102" s="5"/>
+      <c r="B102" s="5"/>
+      <c r="C102" s="5"/>
+    </row>
+    <row r="103" ht="15" customHeight="1">
+      <c r="A103" s="5"/>
+      <c r="B103" s="5"/>
+      <c r="C103" s="5"/>
+    </row>
+    <row r="104" ht="15" customHeight="1">
+      <c r="A104" s="5"/>
+      <c r="B104" s="5"/>
+      <c r="C104" s="5"/>
+    </row>
+    <row r="105" ht="15" customHeight="1">
+      <c r="A105" s="5"/>
+      <c r="B105" s="5"/>
+      <c r="C105" s="5"/>
+    </row>
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" s="5"/>
+      <c r="B106" s="5"/>
+      <c r="C106" s="5"/>
+    </row>
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" s="5"/>
+      <c r="B107" s="5"/>
+      <c r="C107" s="5"/>
+    </row>
+    <row r="108" ht="15" customHeight="1">
+      <c r="A108" s="5"/>
+      <c r="B108" s="5"/>
+      <c r="C108" s="5"/>
+    </row>
+    <row r="109" ht="15" customHeight="1">
+      <c r="A109" s="5"/>
+      <c r="B109" s="5"/>
+      <c r="C109" s="5"/>
+    </row>
+    <row r="110" ht="15" customHeight="1">
+      <c r="A110" s="5"/>
+      <c r="B110" s="5"/>
+      <c r="C110" s="5"/>
+    </row>
+    <row r="111" ht="15" customHeight="1">
+      <c r="A111" s="5"/>
+      <c r="B111" s="5"/>
+      <c r="C111" s="5"/>
+    </row>
+    <row r="112" ht="15" customHeight="1">
+      <c r="A112" s="5"/>
+      <c r="B112" s="5"/>
+      <c r="C112" s="5"/>
+    </row>
+    <row r="113" ht="15" customHeight="1">
+      <c r="A113" s="5"/>
+      <c r="B113" s="5"/>
+      <c r="C113" s="5"/>
+    </row>
+    <row r="114" ht="15" customHeight="1">
+      <c r="A114" s="5"/>
+      <c r="B114" s="5"/>
+      <c r="C114" s="5"/>
+    </row>
+    <row r="115" ht="15" customHeight="1">
+      <c r="A115" s="5"/>
+      <c r="B115" s="5"/>
+      <c r="C115" s="5"/>
+    </row>
+    <row r="116" ht="15" customHeight="1">
+      <c r="A116" s="5"/>
+      <c r="B116" s="5"/>
+      <c r="C116" s="5"/>
+    </row>
+    <row r="117" ht="15" customHeight="1">
+      <c r="A117" s="5"/>
+      <c r="B117" s="5"/>
+      <c r="C117" s="5"/>
+    </row>
+    <row r="118" ht="15" customHeight="1">
+      <c r="A118" s="5"/>
+      <c r="B118" s="5"/>
+      <c r="C118" s="5"/>
+    </row>
+    <row r="119" ht="15" customHeight="1">
+      <c r="A119" s="5"/>
+      <c r="B119" s="5"/>
+      <c r="C119" s="5"/>
+    </row>
+    <row r="120" ht="15" customHeight="1">
+      <c r="A120" s="5"/>
+      <c r="B120" s="5"/>
+      <c r="C120" s="5"/>
+    </row>
+    <row r="121" ht="15" customHeight="1">
+      <c r="A121" s="5"/>
+      <c r="B121" s="5"/>
+      <c r="C121" s="5"/>
+    </row>
+    <row r="122" ht="15" customHeight="1">
+      <c r="A122" s="5"/>
+      <c r="B122" s="5"/>
+      <c r="C122" s="5"/>
+    </row>
+    <row r="123" ht="15" customHeight="1">
+      <c r="A123" s="5"/>
+      <c r="B123" s="5"/>
+      <c r="C123" s="5"/>
+    </row>
+    <row r="124" ht="15" customHeight="1">
+      <c r="A124" s="5"/>
+      <c r="B124" s="5"/>
+      <c r="C124" s="5"/>
+    </row>
+    <row r="125" ht="15" customHeight="1">
+      <c r="A125" s="5"/>
+      <c r="B125" s="5"/>
+      <c r="C125" s="5"/>
+    </row>
+    <row r="126" ht="15" customHeight="1">
+      <c r="A126" s="5"/>
+      <c r="B126" s="5"/>
+      <c r="C126" s="5"/>
+    </row>
+    <row r="127" ht="15" customHeight="1">
+      <c r="A127" s="5"/>
+      <c r="B127" s="5"/>
+      <c r="C127" s="5"/>
+    </row>
+    <row r="128" ht="15" customHeight="1">
+      <c r="A128" s="5"/>
+      <c r="B128" s="5"/>
+      <c r="C128" s="5"/>
+    </row>
+    <row r="129" ht="15" customHeight="1">
+      <c r="A129" s="5"/>
+      <c r="B129" s="5"/>
+      <c r="C129" s="5"/>
+    </row>
+    <row r="130" ht="15" customHeight="1">
+      <c r="A130" s="5"/>
+      <c r="B130" s="5"/>
+      <c r="C130" s="5"/>
+    </row>
+    <row r="131" ht="15" customHeight="1">
+      <c r="A131" s="5"/>
+      <c r="B131" s="5"/>
+      <c r="C131" s="5"/>
+    </row>
+    <row r="132" ht="15" customHeight="1">
+      <c r="A132" s="5"/>
+      <c r="B132" s="5"/>
+      <c r="C132" s="5"/>
+    </row>
+    <row r="133" ht="15" customHeight="1">
+      <c r="A133" s="5"/>
+      <c r="B133" s="5"/>
+      <c r="C133" s="5"/>
+    </row>
+    <row r="134" ht="15" customHeight="1">
+      <c r="A134" s="5"/>
+      <c r="B134" s="5"/>
+      <c r="C134" s="5"/>
+    </row>
+    <row r="135" ht="15" customHeight="1">
+      <c r="A135" s="5"/>
+      <c r="B135" s="5"/>
+      <c r="C135" s="5"/>
+    </row>
+    <row r="136" ht="15" customHeight="1">
+      <c r="A136" s="5"/>
+      <c r="B136" s="5"/>
+      <c r="C136" s="5"/>
+    </row>
+    <row r="137" ht="15" customHeight="1">
+      <c r="A137" s="5"/>
+      <c r="B137" s="5"/>
+      <c r="C137" s="5"/>
+    </row>
+    <row r="138" ht="15" customHeight="1">
+      <c r="A138" s="5"/>
+      <c r="B138" s="5"/>
+      <c r="C138" s="5"/>
+    </row>
+    <row r="139" ht="15" customHeight="1">
+      <c r="A139" s="5"/>
+      <c r="B139" s="5"/>
+      <c r="C139" s="5"/>
+    </row>
+    <row r="140" ht="15" customHeight="1">
+      <c r="A140" s="5"/>
+      <c r="B140" s="5"/>
+      <c r="C140" s="5"/>
+    </row>
+    <row r="141" ht="15" customHeight="1">
+      <c r="A141" s="5"/>
+      <c r="B141" s="5"/>
+      <c r="C141" s="5"/>
+    </row>
+    <row r="142" ht="15" customHeight="1">
+      <c r="A142" s="5"/>
+      <c r="B142" s="5"/>
+      <c r="C142" s="5"/>
+    </row>
+    <row r="143" ht="15" customHeight="1">
+      <c r="A143" s="5"/>
+      <c r="B143" s="5"/>
+      <c r="C143" s="5"/>
+    </row>
+    <row r="144" ht="15" customHeight="1">
+      <c r="A144" s="5"/>
+      <c r="B144" s="5"/>
+      <c r="C144" s="5"/>
+    </row>
+    <row r="145" ht="15" customHeight="1">
+      <c r="A145" s="5"/>
+      <c r="B145" s="5"/>
+      <c r="C145" s="5"/>
+    </row>
+    <row r="146" ht="15" customHeight="1">
+      <c r="A146" s="5"/>
+      <c r="B146" s="5"/>
+      <c r="C146" s="5"/>
+    </row>
+    <row r="147" ht="15" customHeight="1">
+      <c r="A147" s="5"/>
+      <c r="B147" s="5"/>
+      <c r="C147" s="5"/>
+    </row>
+    <row r="148" ht="15" customHeight="1">
+      <c r="A148" s="5"/>
+      <c r="B148" s="5"/>
+      <c r="C148" s="5"/>
+    </row>
+    <row r="149" ht="15" customHeight="1">
+      <c r="A149" s="5"/>
+      <c r="B149" s="5"/>
+      <c r="C149" s="5"/>
+    </row>
+    <row r="150" ht="15" customHeight="1">
+      <c r="A150" s="5"/>
+      <c r="B150" s="5"/>
+      <c r="C150" s="5"/>
+    </row>
+    <row r="151" ht="15" customHeight="1">
+      <c r="A151" s="5"/>
+      <c r="B151" s="5"/>
+      <c r="C151" s="5"/>
+    </row>
+    <row r="152" ht="15" customHeight="1">
+      <c r="A152" s="5"/>
+      <c r="B152" s="5"/>
+      <c r="C152" s="5"/>
+    </row>
+    <row r="153" ht="15" customHeight="1">
+      <c r="A153" s="5"/>
+      <c r="B153" s="5"/>
+      <c r="C153" s="5"/>
+    </row>
+    <row r="154" ht="15" customHeight="1">
+      <c r="A154" s="5"/>
+      <c r="B154" s="5"/>
+      <c r="C154" s="5"/>
+    </row>
+    <row r="155" ht="15" customHeight="1">
+      <c r="A155" s="5"/>
+      <c r="B155" s="5"/>
+      <c r="C155" s="5"/>
+    </row>
+    <row r="156" ht="15" customHeight="1">
+      <c r="A156" s="5"/>
+      <c r="B156" s="5"/>
+      <c r="C156" s="5"/>
+    </row>
+    <row r="157" ht="15" customHeight="1">
+      <c r="A157" s="5"/>
+      <c r="B157" s="5"/>
+      <c r="C157" s="5"/>
+    </row>
+    <row r="158" ht="15" customHeight="1">
+      <c r="A158" s="5"/>
+      <c r="B158" s="5"/>
+      <c r="C158" s="5"/>
+    </row>
+    <row r="159" ht="15" customHeight="1">
+      <c r="A159" s="5"/>
+      <c r="B159" s="5"/>
+      <c r="C159" s="5"/>
+    </row>
+    <row r="160" ht="15" customHeight="1">
+      <c r="A160" s="5"/>
+      <c r="B160" s="5"/>
+      <c r="C160" s="5"/>
+    </row>
+    <row r="161" ht="15" customHeight="1">
+      <c r="A161" s="5"/>
+      <c r="B161" s="5"/>
+      <c r="C161" s="5"/>
+    </row>
+    <row r="162" ht="15" customHeight="1">
+      <c r="A162" s="5"/>
+      <c r="B162" s="5"/>
+      <c r="C162" s="5"/>
+    </row>
+    <row r="163" ht="15" customHeight="1">
+      <c r="A163" s="5"/>
+      <c r="B163" s="5"/>
+      <c r="C163" s="5"/>
+    </row>
+    <row r="164" ht="15" customHeight="1">
+      <c r="A164" s="5"/>
+      <c r="B164" s="5"/>
+      <c r="C164" s="5"/>
+    </row>
+    <row r="165" ht="15" customHeight="1">
+      <c r="A165" s="5"/>
+      <c r="B165" s="5"/>
+      <c r="C165" s="5"/>
+    </row>
+    <row r="166" ht="15" customHeight="1">
+      <c r="A166" s="5"/>
+      <c r="B166" s="5"/>
+      <c r="C166" s="5"/>
+    </row>
+    <row r="167" ht="15" customHeight="1">
+      <c r="A167" s="5"/>
+      <c r="B167" s="5"/>
+      <c r="C167" s="5"/>
+    </row>
+    <row r="168" ht="15" customHeight="1">
+      <c r="A168" s="5"/>
+      <c r="B168" s="5"/>
+      <c r="C168" s="5"/>
+    </row>
+    <row r="169" ht="15" customHeight="1">
+      <c r="A169" s="5"/>
+      <c r="B169" s="5"/>
+      <c r="C169" s="5"/>
+    </row>
+    <row r="170" ht="15" customHeight="1">
+      <c r="A170" s="5"/>
+      <c r="B170" s="5"/>
+      <c r="C170" s="5"/>
+    </row>
+    <row r="171" ht="15" customHeight="1">
+      <c r="A171" s="5"/>
+      <c r="B171" s="5"/>
+      <c r="C171" s="5"/>
+    </row>
+    <row r="172" ht="15" customHeight="1">
+      <c r="A172" s="5"/>
+      <c r="B172" s="5"/>
+      <c r="C172" s="5"/>
+    </row>
+    <row r="173" ht="15" customHeight="1">
+      <c r="A173" s="5"/>
+      <c r="B173" s="5"/>
+      <c r="C173" s="5"/>
+    </row>
+    <row r="174" ht="15" customHeight="1">
+      <c r="A174" s="5"/>
+      <c r="B174" s="5"/>
+      <c r="C174" s="5"/>
+    </row>
+    <row r="175" ht="15" customHeight="1">
+      <c r="A175" s="5"/>
+      <c r="B175" s="5"/>
+      <c r="C175" s="5"/>
+    </row>
+    <row r="176" ht="15" customHeight="1">
+      <c r="A176" s="5"/>
+      <c r="B176" s="5"/>
+      <c r="C176" s="5"/>
+    </row>
+    <row r="177" ht="15" customHeight="1">
+      <c r="A177" s="5"/>
+      <c r="B177" s="5"/>
+      <c r="C177" s="5"/>
+    </row>
+    <row r="178" ht="15" customHeight="1">
+      <c r="A178" s="5"/>
+      <c r="B178" s="5"/>
+      <c r="C178" s="5"/>
+    </row>
+    <row r="179" ht="15" customHeight="1">
+      <c r="A179" s="5"/>
+      <c r="B179" s="5"/>
+      <c r="C179" s="5"/>
+    </row>
+    <row r="180" ht="15" customHeight="1">
+      <c r="A180" s="5"/>
+      <c r="B180" s="5"/>
+      <c r="C180" s="5"/>
+    </row>
+    <row r="181" ht="15" customHeight="1">
+      <c r="A181" s="5"/>
+      <c r="B181" s="5"/>
+      <c r="C181" s="5"/>
+    </row>
+    <row r="182" ht="15" customHeight="1">
+      <c r="A182" s="5"/>
+      <c r="B182" s="5"/>
+      <c r="C182" s="5"/>
+    </row>
+    <row r="183" ht="15" customHeight="1">
+      <c r="A183" s="5"/>
+      <c r="B183" s="5"/>
+      <c r="C183" s="5"/>
+    </row>
+    <row r="184" ht="15" customHeight="1">
+      <c r="A184" s="5"/>
+      <c r="B184" s="5"/>
+      <c r="C184" s="5"/>
+    </row>
+    <row r="185" ht="15" customHeight="1">
+      <c r="A185" s="5"/>
+      <c r="B185" s="5"/>
+      <c r="C185" s="5"/>
+    </row>
+    <row r="186" ht="15" customHeight="1">
+      <c r="A186" s="5"/>
+      <c r="B186" s="5"/>
+      <c r="C186" s="5"/>
+    </row>
+    <row r="187" ht="15" customHeight="1">
+      <c r="A187" s="5"/>
+      <c r="B187" s="5"/>
+      <c r="C187" s="5"/>
+    </row>
+    <row r="188" ht="15" customHeight="1">
+      <c r="A188" s="5"/>
+      <c r="B188" s="5"/>
+      <c r="C188" s="5"/>
+    </row>
+    <row r="189" ht="15" customHeight="1">
+      <c r="A189" s="5"/>
+      <c r="B189" s="5"/>
+      <c r="C189" s="5"/>
+    </row>
+    <row r="190" ht="15" customHeight="1">
+      <c r="A190" s="5"/>
+      <c r="B190" s="5"/>
+      <c r="C190" s="5"/>
+    </row>
+    <row r="191" ht="15" customHeight="1">
+      <c r="A191" s="5"/>
+      <c r="B191" s="5"/>
+      <c r="C191" s="5"/>
+    </row>
+    <row r="192" ht="15" customHeight="1">
+      <c r="A192" s="5"/>
+      <c r="B192" s="5"/>
+      <c r="C192" s="5"/>
+    </row>
+    <row r="193" ht="15" customHeight="1">
+      <c r="A193" s="5"/>
+      <c r="B193" s="5"/>
+      <c r="C193" s="5"/>
+    </row>
+    <row r="194" ht="15" customHeight="1">
+      <c r="A194" s="5"/>
+      <c r="B194" s="5"/>
+      <c r="C194" s="5"/>
+    </row>
+    <row r="195" ht="15" customHeight="1">
+      <c r="A195" s="5"/>
+      <c r="B195" s="5"/>
+      <c r="C195" s="5"/>
+    </row>
+    <row r="196" ht="15" customHeight="1">
+      <c r="A196" s="5"/>
+      <c r="B196" s="5"/>
+      <c r="C196" s="5"/>
+    </row>
+    <row r="197" ht="15" customHeight="1">
+      <c r="A197" s="5"/>
+      <c r="B197" s="5"/>
+      <c r="C197" s="5"/>
+    </row>
+    <row r="198" ht="15" customHeight="1">
+      <c r="A198" s="5"/>
+      <c r="B198" s="5"/>
+      <c r="C198" s="5"/>
+    </row>
+    <row r="199" ht="15" customHeight="1">
+      <c r="A199" s="5"/>
+      <c r="B199" s="5"/>
+      <c r="C199" s="5"/>
+    </row>
+    <row r="200" ht="15" customHeight="1">
+      <c r="A200" s="5"/>
+      <c r="B200" s="5"/>
+      <c r="C200" s="5"/>
+    </row>
+    <row r="201" ht="15" customHeight="1">
+      <c r="A201" s="5"/>
+      <c r="B201" s="5"/>
+      <c r="C201" s="5"/>
+    </row>
+    <row r="202" ht="15" customHeight="1">
+      <c r="A202" s="5"/>
+      <c r="B202" s="5"/>
+      <c r="C202" s="5"/>
+    </row>
+    <row r="203" ht="15" customHeight="1">
+      <c r="A203" s="5"/>
+      <c r="B203" s="5"/>
+      <c r="C203" s="5"/>
+    </row>
+    <row r="204" ht="15" customHeight="1">
+      <c r="A204" s="5"/>
+      <c r="B204" s="5"/>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>

<commit_message>
Implemented defender selling with 50% energy refund
When recalling a defender they will be refunded half the price you spend on, so Shooter is 100 meaning you will get 50 energy back
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView activeTab="4"/>
+    <workbookView activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Enemies" sheetId="1"/>
@@ -114,9 +114,6 @@
     <t>landmine</t>
   </si>
   <si>
-    <t>.</t>
-  </si>
-  <si>
     <t>setting</t>
   </si>
   <si>
@@ -148,6 +145,9 @@
   </si>
   <si>
     <t>passive_energy_interval_ms</t>
+  </si>
+  <si>
+    <t>sell_refund_multiplier</t>
   </si>
   <si>
     <t>starting_health</t>
@@ -311,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment vertical="top"/>
@@ -320,7 +320,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -617,7 +616,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{17B26627-4658-1E69-E178-79CD8F678468}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{49210968-6DA8-10F8-A4F7-5E35F5FBF9E3}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -824,7 +823,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3A4775A7-619D-FD08-96FE-A3BF007A5057}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E5A228F5-2A9E-9C58-0299-9BDDBF263681}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1199,9 +1198,7 @@
       <c r="A8" s="2"/>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="M18" s="4" t="s">
-        <v>32</v>
-      </c>
+      <c r="M18" s="2"/>
     </row>
   </sheetData>
   <printOptions/>
@@ -1216,7 +1213,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9A67F351-5B48-7EB4-C418-995218B62B61}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{34C27081-BB78-FD58-8FA3-A770F9D16E78}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1225,15 +1222,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1241,7 +1238,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1249,7 +1246,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1257,7 +1254,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1265,7 +1262,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1273,7 +1270,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1281,7 +1278,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1289,7 +1286,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1297,10 +1294,18 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="4">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -1316,7 +1321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{541411E8-C1A8-1FB8-09D8-0ED3EA313A87}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4F8B48F8-4D48-1359-B348-545E7A68C828}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1325,10 +1330,10 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
@@ -1368,7 +1373,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B7220D78-D478-C2BF-79C8-39C007D22C68}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{47E5742A-B698-6868-8BC3-10E749DFCCFD}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T204"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1377,10 +1382,10 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
@@ -1416,21 +1421,21 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="2">
         <v>0.15</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <v>0.15</v>
       </c>
-      <c r="C7" s="5"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
@@ -1439,7 +1444,7 @@
       <c r="B8" s="2">
         <v>0.1</v>
       </c>
-      <c r="C8" s="5"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
@@ -1448,7 +1453,7 @@
       <c r="B9" s="2">
         <v>1</v>
       </c>
-      <c r="C9" s="5"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
@@ -1457,7 +1462,7 @@
       <c r="B10" s="2">
         <v>3</v>
       </c>
-      <c r="C10" s="5"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
@@ -1466,7 +1471,7 @@
       <c r="B11" s="2">
         <v>2</v>
       </c>
-      <c r="C11" s="5"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
@@ -1475,7 +1480,7 @@
       <c r="B12" s="2">
         <v>3</v>
       </c>
-      <c r="C12" s="5"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
@@ -1484,7 +1489,7 @@
       <c r="B13" s="2">
         <v>3</v>
       </c>
-      <c r="C13" s="5"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
@@ -1493,7 +1498,7 @@
       <c r="B14" s="2">
         <v>3</v>
       </c>
-      <c r="C14" s="5"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
@@ -1502,7 +1507,7 @@
       <c r="B15" s="2">
         <v>5</v>
       </c>
-      <c r="C15" s="5"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
@@ -1511,25 +1516,25 @@
       <c r="B16" s="2">
         <v>10</v>
       </c>
-      <c r="C16" s="5"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <v>15</v>
       </c>
-      <c r="C17" s="5"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <v>10</v>
       </c>
-      <c r="C18" s="5"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
@@ -1538,7 +1543,7 @@
       <c r="B19" s="2">
         <v>20</v>
       </c>
-      <c r="C19" s="5"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
@@ -1547,7 +1552,7 @@
       <c r="B20" s="2">
         <v>15</v>
       </c>
-      <c r="C20" s="5"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
@@ -1556,7 +1561,7 @@
       <c r="B21" s="2">
         <v>20</v>
       </c>
-      <c r="C21" s="5"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
@@ -1565,7 +1570,7 @@
       <c r="B22" s="2">
         <v>30</v>
       </c>
-      <c r="C22" s="5"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
@@ -1574,7 +1579,7 @@
       <c r="B23" s="2">
         <v>40</v>
       </c>
-      <c r="C23" s="5"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
@@ -1583,7 +1588,7 @@
       <c r="B24" s="2">
         <v>50</v>
       </c>
-      <c r="C24" s="5"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
@@ -1592,7 +1597,7 @@
       <c r="B25" s="2">
         <v>60</v>
       </c>
-      <c r="C25" s="5"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
@@ -1601,7 +1606,7 @@
       <c r="B26" s="2">
         <v>50</v>
       </c>
-      <c r="C26" s="5"/>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
@@ -1610,7 +1615,7 @@
       <c r="B27" s="2">
         <v>65</v>
       </c>
-      <c r="C27" s="5"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
@@ -1619,7 +1624,7 @@
       <c r="B28" s="2">
         <v>80</v>
       </c>
-      <c r="C28" s="5"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="2" t="s">
@@ -1628,7 +1633,7 @@
       <c r="B29" s="2">
         <v>70</v>
       </c>
-      <c r="C29" s="5"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="2" t="s">
@@ -1637,7 +1642,7 @@
       <c r="B30" s="2">
         <v>90</v>
       </c>
-      <c r="C30" s="5"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="2" t="s">
@@ -1646,7 +1651,7 @@
       <c r="B31" s="2">
         <v>110</v>
       </c>
-      <c r="C31" s="5"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="2" t="s">
@@ -1655,874 +1660,874 @@
       <c r="B32" s="2">
         <v>10000</v>
       </c>
-      <c r="C32" s="5"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33" s="2">
         <v>0.1</v>
       </c>
-      <c r="C33" s="5"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34" s="2">
         <v>0.05</v>
       </c>
-      <c r="C34" s="5"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="5"/>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
     </row>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
     </row>
     <row r="42" ht="15" customHeight="1">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5"/>
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
     </row>
     <row r="44" ht="15" customHeight="1">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5"/>
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
     </row>
     <row r="45" ht="15" customHeight="1">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
     </row>
     <row r="46" ht="15" customHeight="1">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
-      <c r="C46" s="5"/>
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
-      <c r="C47" s="5"/>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
     </row>
     <row r="48" ht="15" customHeight="1">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="5"/>
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
-      <c r="C50" s="5"/>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="5"/>
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
     </row>
     <row r="53" ht="15" customHeight="1">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
-      <c r="C53" s="5"/>
+      <c r="A53" s="2"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
     </row>
     <row r="54" ht="15" customHeight="1">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
-      <c r="C54" s="5"/>
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
     </row>
     <row r="55" ht="15" customHeight="1">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
     </row>
     <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5"/>
-      <c r="C57" s="5"/>
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
     </row>
     <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
     </row>
     <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
     </row>
     <row r="60" ht="15" customHeight="1">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
     </row>
     <row r="61" ht="15" customHeight="1">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
     </row>
     <row r="62" ht="15" customHeight="1">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
     </row>
     <row r="63" ht="15" customHeight="1">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
     </row>
     <row r="64" ht="15" customHeight="1">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
-      <c r="C64" s="5"/>
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
     </row>
     <row r="65" ht="15" customHeight="1">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
-      <c r="C65" s="5"/>
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
     </row>
     <row r="66" ht="15" customHeight="1">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5"/>
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
     </row>
     <row r="67" ht="15" customHeight="1">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
     </row>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="C68" s="5"/>
+      <c r="A68" s="2"/>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
     </row>
     <row r="69" ht="15" customHeight="1">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
     </row>
     <row r="70" ht="15" customHeight="1">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
-      <c r="C70" s="5"/>
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
     </row>
     <row r="71" ht="15" customHeight="1">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="C71" s="5"/>
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
     </row>
     <row r="72" ht="15" customHeight="1">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5"/>
-      <c r="C72" s="5"/>
+      <c r="A72" s="2"/>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
     </row>
     <row r="73" ht="15" customHeight="1">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
-      <c r="C73" s="5"/>
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
-      <c r="C74" s="5"/>
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2"/>
     </row>
     <row r="75" ht="15" customHeight="1">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
-      <c r="C75" s="5"/>
+      <c r="A75" s="2"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
     </row>
     <row r="76" ht="15" customHeight="1">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
+      <c r="A76" s="2"/>
+      <c r="B76" s="2"/>
+      <c r="C76" s="2"/>
     </row>
     <row r="77" ht="15" customHeight="1">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5"/>
-      <c r="C77" s="5"/>
+      <c r="A77" s="2"/>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
     </row>
     <row r="78" ht="15" customHeight="1">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
-      <c r="C78" s="5"/>
+      <c r="A78" s="2"/>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2"/>
     </row>
     <row r="79" ht="15" customHeight="1">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
-      <c r="C79" s="5"/>
+      <c r="A79" s="2"/>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2"/>
     </row>
     <row r="80" ht="15" customHeight="1">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
-      <c r="C80" s="5"/>
+      <c r="A80" s="2"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
     </row>
     <row r="81" ht="15" customHeight="1">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
-      <c r="C81" s="5"/>
+      <c r="A81" s="2"/>
+      <c r="B81" s="2"/>
+      <c r="C81" s="2"/>
     </row>
     <row r="82" ht="15" customHeight="1">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5"/>
-      <c r="C82" s="5"/>
+      <c r="A82" s="2"/>
+      <c r="B82" s="2"/>
+      <c r="C82" s="2"/>
     </row>
     <row r="83" ht="15" customHeight="1">
-      <c r="A83" s="5"/>
-      <c r="B83" s="5"/>
-      <c r="C83" s="5"/>
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2"/>
     </row>
     <row r="84" ht="15" customHeight="1">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
-      <c r="C84" s="5"/>
+      <c r="A84" s="2"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2"/>
     </row>
     <row r="85" ht="15" customHeight="1">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
-      <c r="C85" s="5"/>
+      <c r="A85" s="2"/>
+      <c r="B85" s="2"/>
+      <c r="C85" s="2"/>
     </row>
     <row r="86" ht="15" customHeight="1">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
-      <c r="C86" s="5"/>
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="2"/>
     </row>
     <row r="87" ht="15" customHeight="1">
-      <c r="A87" s="5"/>
-      <c r="B87" s="5"/>
-      <c r="C87" s="5"/>
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="2"/>
     </row>
     <row r="88" ht="15" customHeight="1">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
-      <c r="C88" s="5"/>
+      <c r="A88" s="2"/>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2"/>
     </row>
     <row r="89" ht="15" customHeight="1">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
-      <c r="C89" s="5"/>
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="2"/>
     </row>
     <row r="90" ht="15" customHeight="1">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
-      <c r="C90" s="5"/>
+      <c r="A90" s="2"/>
+      <c r="B90" s="2"/>
+      <c r="C90" s="2"/>
     </row>
     <row r="91" ht="15" customHeight="1">
-      <c r="A91" s="5"/>
-      <c r="B91" s="5"/>
-      <c r="C91" s="5"/>
+      <c r="A91" s="2"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2"/>
     </row>
     <row r="92" ht="15" customHeight="1">
-      <c r="A92" s="5"/>
-      <c r="B92" s="5"/>
-      <c r="C92" s="5"/>
+      <c r="A92" s="2"/>
+      <c r="B92" s="2"/>
+      <c r="C92" s="2"/>
     </row>
     <row r="93" ht="15" customHeight="1">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
-      <c r="C93" s="5"/>
+      <c r="A93" s="2"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
     </row>
     <row r="94" ht="15" customHeight="1">
-      <c r="A94" s="5"/>
-      <c r="B94" s="5"/>
-      <c r="C94" s="5"/>
+      <c r="A94" s="2"/>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2"/>
     </row>
     <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="5"/>
-      <c r="B95" s="5"/>
-      <c r="C95" s="5"/>
+      <c r="A95" s="2"/>
+      <c r="B95" s="2"/>
+      <c r="C95" s="2"/>
     </row>
     <row r="96" ht="15" customHeight="1">
-      <c r="A96" s="5"/>
-      <c r="B96" s="5"/>
-      <c r="C96" s="5"/>
+      <c r="A96" s="2"/>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2"/>
     </row>
     <row r="97" ht="15" customHeight="1">
-      <c r="A97" s="5"/>
-      <c r="B97" s="5"/>
-      <c r="C97" s="5"/>
+      <c r="A97" s="2"/>
+      <c r="B97" s="2"/>
+      <c r="C97" s="2"/>
     </row>
     <row r="98" ht="15" customHeight="1">
-      <c r="A98" s="5"/>
-      <c r="B98" s="5"/>
-      <c r="C98" s="5"/>
+      <c r="A98" s="2"/>
+      <c r="B98" s="2"/>
+      <c r="C98" s="2"/>
     </row>
     <row r="99" ht="15" customHeight="1">
-      <c r="A99" s="5"/>
-      <c r="B99" s="5"/>
-      <c r="C99" s="5"/>
+      <c r="A99" s="2"/>
+      <c r="B99" s="2"/>
+      <c r="C99" s="2"/>
     </row>
     <row r="100" ht="15" customHeight="1">
-      <c r="A100" s="5"/>
-      <c r="B100" s="5"/>
-      <c r="C100" s="5"/>
+      <c r="A100" s="2"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
     </row>
     <row r="101" ht="15" customHeight="1">
-      <c r="A101" s="5"/>
-      <c r="B101" s="5"/>
-      <c r="C101" s="5"/>
+      <c r="A101" s="2"/>
+      <c r="B101" s="2"/>
+      <c r="C101" s="2"/>
     </row>
     <row r="102" ht="15" customHeight="1">
-      <c r="A102" s="5"/>
-      <c r="B102" s="5"/>
-      <c r="C102" s="5"/>
+      <c r="A102" s="2"/>
+      <c r="B102" s="2"/>
+      <c r="C102" s="2"/>
     </row>
     <row r="103" ht="15" customHeight="1">
-      <c r="A103" s="5"/>
-      <c r="B103" s="5"/>
-      <c r="C103" s="5"/>
+      <c r="A103" s="2"/>
+      <c r="B103" s="2"/>
+      <c r="C103" s="2"/>
     </row>
     <row r="104" ht="15" customHeight="1">
-      <c r="A104" s="5"/>
-      <c r="B104" s="5"/>
-      <c r="C104" s="5"/>
+      <c r="A104" s="2"/>
+      <c r="B104" s="2"/>
+      <c r="C104" s="2"/>
     </row>
     <row r="105" ht="15" customHeight="1">
-      <c r="A105" s="5"/>
-      <c r="B105" s="5"/>
-      <c r="C105" s="5"/>
+      <c r="A105" s="2"/>
+      <c r="B105" s="2"/>
+      <c r="C105" s="2"/>
     </row>
     <row r="106" ht="15" customHeight="1">
-      <c r="A106" s="5"/>
-      <c r="B106" s="5"/>
-      <c r="C106" s="5"/>
+      <c r="A106" s="2"/>
+      <c r="B106" s="2"/>
+      <c r="C106" s="2"/>
     </row>
     <row r="107" ht="15" customHeight="1">
-      <c r="A107" s="5"/>
-      <c r="B107" s="5"/>
-      <c r="C107" s="5"/>
+      <c r="A107" s="2"/>
+      <c r="B107" s="2"/>
+      <c r="C107" s="2"/>
     </row>
     <row r="108" ht="15" customHeight="1">
-      <c r="A108" s="5"/>
-      <c r="B108" s="5"/>
-      <c r="C108" s="5"/>
+      <c r="A108" s="2"/>
+      <c r="B108" s="2"/>
+      <c r="C108" s="2"/>
     </row>
     <row r="109" ht="15" customHeight="1">
-      <c r="A109" s="5"/>
-      <c r="B109" s="5"/>
-      <c r="C109" s="5"/>
+      <c r="A109" s="2"/>
+      <c r="B109" s="2"/>
+      <c r="C109" s="2"/>
     </row>
     <row r="110" ht="15" customHeight="1">
-      <c r="A110" s="5"/>
-      <c r="B110" s="5"/>
-      <c r="C110" s="5"/>
+      <c r="A110" s="2"/>
+      <c r="B110" s="2"/>
+      <c r="C110" s="2"/>
     </row>
     <row r="111" ht="15" customHeight="1">
-      <c r="A111" s="5"/>
-      <c r="B111" s="5"/>
-      <c r="C111" s="5"/>
+      <c r="A111" s="2"/>
+      <c r="B111" s="2"/>
+      <c r="C111" s="2"/>
     </row>
     <row r="112" ht="15" customHeight="1">
-      <c r="A112" s="5"/>
-      <c r="B112" s="5"/>
-      <c r="C112" s="5"/>
+      <c r="A112" s="2"/>
+      <c r="B112" s="2"/>
+      <c r="C112" s="2"/>
     </row>
     <row r="113" ht="15" customHeight="1">
-      <c r="A113" s="5"/>
-      <c r="B113" s="5"/>
-      <c r="C113" s="5"/>
+      <c r="A113" s="2"/>
+      <c r="B113" s="2"/>
+      <c r="C113" s="2"/>
     </row>
     <row r="114" ht="15" customHeight="1">
-      <c r="A114" s="5"/>
-      <c r="B114" s="5"/>
-      <c r="C114" s="5"/>
+      <c r="A114" s="2"/>
+      <c r="B114" s="2"/>
+      <c r="C114" s="2"/>
     </row>
     <row r="115" ht="15" customHeight="1">
-      <c r="A115" s="5"/>
-      <c r="B115" s="5"/>
-      <c r="C115" s="5"/>
+      <c r="A115" s="2"/>
+      <c r="B115" s="2"/>
+      <c r="C115" s="2"/>
     </row>
     <row r="116" ht="15" customHeight="1">
-      <c r="A116" s="5"/>
-      <c r="B116" s="5"/>
-      <c r="C116" s="5"/>
+      <c r="A116" s="2"/>
+      <c r="B116" s="2"/>
+      <c r="C116" s="2"/>
     </row>
     <row r="117" ht="15" customHeight="1">
-      <c r="A117" s="5"/>
-      <c r="B117" s="5"/>
-      <c r="C117" s="5"/>
+      <c r="A117" s="2"/>
+      <c r="B117" s="2"/>
+      <c r="C117" s="2"/>
     </row>
     <row r="118" ht="15" customHeight="1">
-      <c r="A118" s="5"/>
-      <c r="B118" s="5"/>
-      <c r="C118" s="5"/>
+      <c r="A118" s="2"/>
+      <c r="B118" s="2"/>
+      <c r="C118" s="2"/>
     </row>
     <row r="119" ht="15" customHeight="1">
-      <c r="A119" s="5"/>
-      <c r="B119" s="5"/>
-      <c r="C119" s="5"/>
+      <c r="A119" s="2"/>
+      <c r="B119" s="2"/>
+      <c r="C119" s="2"/>
     </row>
     <row r="120" ht="15" customHeight="1">
-      <c r="A120" s="5"/>
-      <c r="B120" s="5"/>
-      <c r="C120" s="5"/>
+      <c r="A120" s="2"/>
+      <c r="B120" s="2"/>
+      <c r="C120" s="2"/>
     </row>
     <row r="121" ht="15" customHeight="1">
-      <c r="A121" s="5"/>
-      <c r="B121" s="5"/>
-      <c r="C121" s="5"/>
+      <c r="A121" s="2"/>
+      <c r="B121" s="2"/>
+      <c r="C121" s="2"/>
     </row>
     <row r="122" ht="15" customHeight="1">
-      <c r="A122" s="5"/>
-      <c r="B122" s="5"/>
-      <c r="C122" s="5"/>
+      <c r="A122" s="2"/>
+      <c r="B122" s="2"/>
+      <c r="C122" s="2"/>
     </row>
     <row r="123" ht="15" customHeight="1">
-      <c r="A123" s="5"/>
-      <c r="B123" s="5"/>
-      <c r="C123" s="5"/>
+      <c r="A123" s="2"/>
+      <c r="B123" s="2"/>
+      <c r="C123" s="2"/>
     </row>
     <row r="124" ht="15" customHeight="1">
-      <c r="A124" s="5"/>
-      <c r="B124" s="5"/>
-      <c r="C124" s="5"/>
+      <c r="A124" s="2"/>
+      <c r="B124" s="2"/>
+      <c r="C124" s="2"/>
     </row>
     <row r="125" ht="15" customHeight="1">
-      <c r="A125" s="5"/>
-      <c r="B125" s="5"/>
-      <c r="C125" s="5"/>
+      <c r="A125" s="2"/>
+      <c r="B125" s="2"/>
+      <c r="C125" s="2"/>
     </row>
     <row r="126" ht="15" customHeight="1">
-      <c r="A126" s="5"/>
-      <c r="B126" s="5"/>
-      <c r="C126" s="5"/>
+      <c r="A126" s="2"/>
+      <c r="B126" s="2"/>
+      <c r="C126" s="2"/>
     </row>
     <row r="127" ht="15" customHeight="1">
-      <c r="A127" s="5"/>
-      <c r="B127" s="5"/>
-      <c r="C127" s="5"/>
+      <c r="A127" s="2"/>
+      <c r="B127" s="2"/>
+      <c r="C127" s="2"/>
     </row>
     <row r="128" ht="15" customHeight="1">
-      <c r="A128" s="5"/>
-      <c r="B128" s="5"/>
-      <c r="C128" s="5"/>
+      <c r="A128" s="2"/>
+      <c r="B128" s="2"/>
+      <c r="C128" s="2"/>
     </row>
     <row r="129" ht="15" customHeight="1">
-      <c r="A129" s="5"/>
-      <c r="B129" s="5"/>
-      <c r="C129" s="5"/>
+      <c r="A129" s="2"/>
+      <c r="B129" s="2"/>
+      <c r="C129" s="2"/>
     </row>
     <row r="130" ht="15" customHeight="1">
-      <c r="A130" s="5"/>
-      <c r="B130" s="5"/>
-      <c r="C130" s="5"/>
+      <c r="A130" s="2"/>
+      <c r="B130" s="2"/>
+      <c r="C130" s="2"/>
     </row>
     <row r="131" ht="15" customHeight="1">
-      <c r="A131" s="5"/>
-      <c r="B131" s="5"/>
-      <c r="C131" s="5"/>
+      <c r="A131" s="2"/>
+      <c r="B131" s="2"/>
+      <c r="C131" s="2"/>
     </row>
     <row r="132" ht="15" customHeight="1">
-      <c r="A132" s="5"/>
-      <c r="B132" s="5"/>
-      <c r="C132" s="5"/>
+      <c r="A132" s="2"/>
+      <c r="B132" s="2"/>
+      <c r="C132" s="2"/>
     </row>
     <row r="133" ht="15" customHeight="1">
-      <c r="A133" s="5"/>
-      <c r="B133" s="5"/>
-      <c r="C133" s="5"/>
+      <c r="A133" s="2"/>
+      <c r="B133" s="2"/>
+      <c r="C133" s="2"/>
     </row>
     <row r="134" ht="15" customHeight="1">
-      <c r="A134" s="5"/>
-      <c r="B134" s="5"/>
-      <c r="C134" s="5"/>
+      <c r="A134" s="2"/>
+      <c r="B134" s="2"/>
+      <c r="C134" s="2"/>
     </row>
     <row r="135" ht="15" customHeight="1">
-      <c r="A135" s="5"/>
-      <c r="B135" s="5"/>
-      <c r="C135" s="5"/>
+      <c r="A135" s="2"/>
+      <c r="B135" s="2"/>
+      <c r="C135" s="2"/>
     </row>
     <row r="136" ht="15" customHeight="1">
-      <c r="A136" s="5"/>
-      <c r="B136" s="5"/>
-      <c r="C136" s="5"/>
+      <c r="A136" s="2"/>
+      <c r="B136" s="2"/>
+      <c r="C136" s="2"/>
     </row>
     <row r="137" ht="15" customHeight="1">
-      <c r="A137" s="5"/>
-      <c r="B137" s="5"/>
-      <c r="C137" s="5"/>
+      <c r="A137" s="2"/>
+      <c r="B137" s="2"/>
+      <c r="C137" s="2"/>
     </row>
     <row r="138" ht="15" customHeight="1">
-      <c r="A138" s="5"/>
-      <c r="B138" s="5"/>
-      <c r="C138" s="5"/>
+      <c r="A138" s="2"/>
+      <c r="B138" s="2"/>
+      <c r="C138" s="2"/>
     </row>
     <row r="139" ht="15" customHeight="1">
-      <c r="A139" s="5"/>
-      <c r="B139" s="5"/>
-      <c r="C139" s="5"/>
+      <c r="A139" s="2"/>
+      <c r="B139" s="2"/>
+      <c r="C139" s="2"/>
     </row>
     <row r="140" ht="15" customHeight="1">
-      <c r="A140" s="5"/>
-      <c r="B140" s="5"/>
-      <c r="C140" s="5"/>
+      <c r="A140" s="2"/>
+      <c r="B140" s="2"/>
+      <c r="C140" s="2"/>
     </row>
     <row r="141" ht="15" customHeight="1">
-      <c r="A141" s="5"/>
-      <c r="B141" s="5"/>
-      <c r="C141" s="5"/>
+      <c r="A141" s="2"/>
+      <c r="B141" s="2"/>
+      <c r="C141" s="2"/>
     </row>
     <row r="142" ht="15" customHeight="1">
-      <c r="A142" s="5"/>
-      <c r="B142" s="5"/>
-      <c r="C142" s="5"/>
+      <c r="A142" s="2"/>
+      <c r="B142" s="2"/>
+      <c r="C142" s="2"/>
     </row>
     <row r="143" ht="15" customHeight="1">
-      <c r="A143" s="5"/>
-      <c r="B143" s="5"/>
-      <c r="C143" s="5"/>
+      <c r="A143" s="2"/>
+      <c r="B143" s="2"/>
+      <c r="C143" s="2"/>
     </row>
     <row r="144" ht="15" customHeight="1">
-      <c r="A144" s="5"/>
-      <c r="B144" s="5"/>
-      <c r="C144" s="5"/>
+      <c r="A144" s="2"/>
+      <c r="B144" s="2"/>
+      <c r="C144" s="2"/>
     </row>
     <row r="145" ht="15" customHeight="1">
-      <c r="A145" s="5"/>
-      <c r="B145" s="5"/>
-      <c r="C145" s="5"/>
+      <c r="A145" s="2"/>
+      <c r="B145" s="2"/>
+      <c r="C145" s="2"/>
     </row>
     <row r="146" ht="15" customHeight="1">
-      <c r="A146" s="5"/>
-      <c r="B146" s="5"/>
-      <c r="C146" s="5"/>
+      <c r="A146" s="2"/>
+      <c r="B146" s="2"/>
+      <c r="C146" s="2"/>
     </row>
     <row r="147" ht="15" customHeight="1">
-      <c r="A147" s="5"/>
-      <c r="B147" s="5"/>
-      <c r="C147" s="5"/>
+      <c r="A147" s="2"/>
+      <c r="B147" s="2"/>
+      <c r="C147" s="2"/>
     </row>
     <row r="148" ht="15" customHeight="1">
-      <c r="A148" s="5"/>
-      <c r="B148" s="5"/>
-      <c r="C148" s="5"/>
+      <c r="A148" s="2"/>
+      <c r="B148" s="2"/>
+      <c r="C148" s="2"/>
     </row>
     <row r="149" ht="15" customHeight="1">
-      <c r="A149" s="5"/>
-      <c r="B149" s="5"/>
-      <c r="C149" s="5"/>
+      <c r="A149" s="2"/>
+      <c r="B149" s="2"/>
+      <c r="C149" s="2"/>
     </row>
     <row r="150" ht="15" customHeight="1">
-      <c r="A150" s="5"/>
-      <c r="B150" s="5"/>
-      <c r="C150" s="5"/>
+      <c r="A150" s="2"/>
+      <c r="B150" s="2"/>
+      <c r="C150" s="2"/>
     </row>
     <row r="151" ht="15" customHeight="1">
-      <c r="A151" s="5"/>
-      <c r="B151" s="5"/>
-      <c r="C151" s="5"/>
+      <c r="A151" s="2"/>
+      <c r="B151" s="2"/>
+      <c r="C151" s="2"/>
     </row>
     <row r="152" ht="15" customHeight="1">
-      <c r="A152" s="5"/>
-      <c r="B152" s="5"/>
-      <c r="C152" s="5"/>
+      <c r="A152" s="2"/>
+      <c r="B152" s="2"/>
+      <c r="C152" s="2"/>
     </row>
     <row r="153" ht="15" customHeight="1">
-      <c r="A153" s="5"/>
-      <c r="B153" s="5"/>
-      <c r="C153" s="5"/>
+      <c r="A153" s="2"/>
+      <c r="B153" s="2"/>
+      <c r="C153" s="2"/>
     </row>
     <row r="154" ht="15" customHeight="1">
-      <c r="A154" s="5"/>
-      <c r="B154" s="5"/>
-      <c r="C154" s="5"/>
+      <c r="A154" s="2"/>
+      <c r="B154" s="2"/>
+      <c r="C154" s="2"/>
     </row>
     <row r="155" ht="15" customHeight="1">
-      <c r="A155" s="5"/>
-      <c r="B155" s="5"/>
-      <c r="C155" s="5"/>
+      <c r="A155" s="2"/>
+      <c r="B155" s="2"/>
+      <c r="C155" s="2"/>
     </row>
     <row r="156" ht="15" customHeight="1">
-      <c r="A156" s="5"/>
-      <c r="B156" s="5"/>
-      <c r="C156" s="5"/>
+      <c r="A156" s="2"/>
+      <c r="B156" s="2"/>
+      <c r="C156" s="2"/>
     </row>
     <row r="157" ht="15" customHeight="1">
-      <c r="A157" s="5"/>
-      <c r="B157" s="5"/>
-      <c r="C157" s="5"/>
+      <c r="A157" s="2"/>
+      <c r="B157" s="2"/>
+      <c r="C157" s="2"/>
     </row>
     <row r="158" ht="15" customHeight="1">
-      <c r="A158" s="5"/>
-      <c r="B158" s="5"/>
-      <c r="C158" s="5"/>
+      <c r="A158" s="2"/>
+      <c r="B158" s="2"/>
+      <c r="C158" s="2"/>
     </row>
     <row r="159" ht="15" customHeight="1">
-      <c r="A159" s="5"/>
-      <c r="B159" s="5"/>
-      <c r="C159" s="5"/>
+      <c r="A159" s="2"/>
+      <c r="B159" s="2"/>
+      <c r="C159" s="2"/>
     </row>
     <row r="160" ht="15" customHeight="1">
-      <c r="A160" s="5"/>
-      <c r="B160" s="5"/>
-      <c r="C160" s="5"/>
+      <c r="A160" s="2"/>
+      <c r="B160" s="2"/>
+      <c r="C160" s="2"/>
     </row>
     <row r="161" ht="15" customHeight="1">
-      <c r="A161" s="5"/>
-      <c r="B161" s="5"/>
-      <c r="C161" s="5"/>
+      <c r="A161" s="2"/>
+      <c r="B161" s="2"/>
+      <c r="C161" s="2"/>
     </row>
     <row r="162" ht="15" customHeight="1">
-      <c r="A162" s="5"/>
-      <c r="B162" s="5"/>
-      <c r="C162" s="5"/>
+      <c r="A162" s="2"/>
+      <c r="B162" s="2"/>
+      <c r="C162" s="2"/>
     </row>
     <row r="163" ht="15" customHeight="1">
-      <c r="A163" s="5"/>
-      <c r="B163" s="5"/>
-      <c r="C163" s="5"/>
+      <c r="A163" s="2"/>
+      <c r="B163" s="2"/>
+      <c r="C163" s="2"/>
     </row>
     <row r="164" ht="15" customHeight="1">
-      <c r="A164" s="5"/>
-      <c r="B164" s="5"/>
-      <c r="C164" s="5"/>
+      <c r="A164" s="2"/>
+      <c r="B164" s="2"/>
+      <c r="C164" s="2"/>
     </row>
     <row r="165" ht="15" customHeight="1">
-      <c r="A165" s="5"/>
-      <c r="B165" s="5"/>
-      <c r="C165" s="5"/>
+      <c r="A165" s="2"/>
+      <c r="B165" s="2"/>
+      <c r="C165" s="2"/>
     </row>
     <row r="166" ht="15" customHeight="1">
-      <c r="A166" s="5"/>
-      <c r="B166" s="5"/>
-      <c r="C166" s="5"/>
+      <c r="A166" s="2"/>
+      <c r="B166" s="2"/>
+      <c r="C166" s="2"/>
     </row>
     <row r="167" ht="15" customHeight="1">
-      <c r="A167" s="5"/>
-      <c r="B167" s="5"/>
-      <c r="C167" s="5"/>
+      <c r="A167" s="2"/>
+      <c r="B167" s="2"/>
+      <c r="C167" s="2"/>
     </row>
     <row r="168" ht="15" customHeight="1">
-      <c r="A168" s="5"/>
-      <c r="B168" s="5"/>
-      <c r="C168" s="5"/>
+      <c r="A168" s="2"/>
+      <c r="B168" s="2"/>
+      <c r="C168" s="2"/>
     </row>
     <row r="169" ht="15" customHeight="1">
-      <c r="A169" s="5"/>
-      <c r="B169" s="5"/>
-      <c r="C169" s="5"/>
+      <c r="A169" s="2"/>
+      <c r="B169" s="2"/>
+      <c r="C169" s="2"/>
     </row>
     <row r="170" ht="15" customHeight="1">
-      <c r="A170" s="5"/>
-      <c r="B170" s="5"/>
-      <c r="C170" s="5"/>
+      <c r="A170" s="2"/>
+      <c r="B170" s="2"/>
+      <c r="C170" s="2"/>
     </row>
     <row r="171" ht="15" customHeight="1">
-      <c r="A171" s="5"/>
-      <c r="B171" s="5"/>
-      <c r="C171" s="5"/>
+      <c r="A171" s="2"/>
+      <c r="B171" s="2"/>
+      <c r="C171" s="2"/>
     </row>
     <row r="172" ht="15" customHeight="1">
-      <c r="A172" s="5"/>
-      <c r="B172" s="5"/>
-      <c r="C172" s="5"/>
+      <c r="A172" s="2"/>
+      <c r="B172" s="2"/>
+      <c r="C172" s="2"/>
     </row>
     <row r="173" ht="15" customHeight="1">
-      <c r="A173" s="5"/>
-      <c r="B173" s="5"/>
-      <c r="C173" s="5"/>
+      <c r="A173" s="2"/>
+      <c r="B173" s="2"/>
+      <c r="C173" s="2"/>
     </row>
     <row r="174" ht="15" customHeight="1">
-      <c r="A174" s="5"/>
-      <c r="B174" s="5"/>
-      <c r="C174" s="5"/>
+      <c r="A174" s="2"/>
+      <c r="B174" s="2"/>
+      <c r="C174" s="2"/>
     </row>
     <row r="175" ht="15" customHeight="1">
-      <c r="A175" s="5"/>
-      <c r="B175" s="5"/>
-      <c r="C175" s="5"/>
+      <c r="A175" s="2"/>
+      <c r="B175" s="2"/>
+      <c r="C175" s="2"/>
     </row>
     <row r="176" ht="15" customHeight="1">
-      <c r="A176" s="5"/>
-      <c r="B176" s="5"/>
-      <c r="C176" s="5"/>
+      <c r="A176" s="2"/>
+      <c r="B176" s="2"/>
+      <c r="C176" s="2"/>
     </row>
     <row r="177" ht="15" customHeight="1">
-      <c r="A177" s="5"/>
-      <c r="B177" s="5"/>
-      <c r="C177" s="5"/>
+      <c r="A177" s="2"/>
+      <c r="B177" s="2"/>
+      <c r="C177" s="2"/>
     </row>
     <row r="178" ht="15" customHeight="1">
-      <c r="A178" s="5"/>
-      <c r="B178" s="5"/>
-      <c r="C178" s="5"/>
+      <c r="A178" s="2"/>
+      <c r="B178" s="2"/>
+      <c r="C178" s="2"/>
     </row>
     <row r="179" ht="15" customHeight="1">
-      <c r="A179" s="5"/>
-      <c r="B179" s="5"/>
-      <c r="C179" s="5"/>
+      <c r="A179" s="2"/>
+      <c r="B179" s="2"/>
+      <c r="C179" s="2"/>
     </row>
     <row r="180" ht="15" customHeight="1">
-      <c r="A180" s="5"/>
-      <c r="B180" s="5"/>
-      <c r="C180" s="5"/>
+      <c r="A180" s="2"/>
+      <c r="B180" s="2"/>
+      <c r="C180" s="2"/>
     </row>
     <row r="181" ht="15" customHeight="1">
-      <c r="A181" s="5"/>
-      <c r="B181" s="5"/>
-      <c r="C181" s="5"/>
+      <c r="A181" s="2"/>
+      <c r="B181" s="2"/>
+      <c r="C181" s="2"/>
     </row>
     <row r="182" ht="15" customHeight="1">
-      <c r="A182" s="5"/>
-      <c r="B182" s="5"/>
-      <c r="C182" s="5"/>
+      <c r="A182" s="2"/>
+      <c r="B182" s="2"/>
+      <c r="C182" s="2"/>
     </row>
     <row r="183" ht="15" customHeight="1">
-      <c r="A183" s="5"/>
-      <c r="B183" s="5"/>
-      <c r="C183" s="5"/>
+      <c r="A183" s="2"/>
+      <c r="B183" s="2"/>
+      <c r="C183" s="2"/>
     </row>
     <row r="184" ht="15" customHeight="1">
-      <c r="A184" s="5"/>
-      <c r="B184" s="5"/>
-      <c r="C184" s="5"/>
+      <c r="A184" s="2"/>
+      <c r="B184" s="2"/>
+      <c r="C184" s="2"/>
     </row>
     <row r="185" ht="15" customHeight="1">
-      <c r="A185" s="5"/>
-      <c r="B185" s="5"/>
-      <c r="C185" s="5"/>
+      <c r="A185" s="2"/>
+      <c r="B185" s="2"/>
+      <c r="C185" s="2"/>
     </row>
     <row r="186" ht="15" customHeight="1">
-      <c r="A186" s="5"/>
-      <c r="B186" s="5"/>
-      <c r="C186" s="5"/>
+      <c r="A186" s="2"/>
+      <c r="B186" s="2"/>
+      <c r="C186" s="2"/>
     </row>
     <row r="187" ht="15" customHeight="1">
-      <c r="A187" s="5"/>
-      <c r="B187" s="5"/>
-      <c r="C187" s="5"/>
+      <c r="A187" s="2"/>
+      <c r="B187" s="2"/>
+      <c r="C187" s="2"/>
     </row>
     <row r="188" ht="15" customHeight="1">
-      <c r="A188" s="5"/>
-      <c r="B188" s="5"/>
-      <c r="C188" s="5"/>
+      <c r="A188" s="2"/>
+      <c r="B188" s="2"/>
+      <c r="C188" s="2"/>
     </row>
     <row r="189" ht="15" customHeight="1">
-      <c r="A189" s="5"/>
-      <c r="B189" s="5"/>
-      <c r="C189" s="5"/>
+      <c r="A189" s="2"/>
+      <c r="B189" s="2"/>
+      <c r="C189" s="2"/>
     </row>
     <row r="190" ht="15" customHeight="1">
-      <c r="A190" s="5"/>
-      <c r="B190" s="5"/>
-      <c r="C190" s="5"/>
+      <c r="A190" s="2"/>
+      <c r="B190" s="2"/>
+      <c r="C190" s="2"/>
     </row>
     <row r="191" ht="15" customHeight="1">
-      <c r="A191" s="5"/>
-      <c r="B191" s="5"/>
-      <c r="C191" s="5"/>
+      <c r="A191" s="2"/>
+      <c r="B191" s="2"/>
+      <c r="C191" s="2"/>
     </row>
     <row r="192" ht="15" customHeight="1">
-      <c r="A192" s="5"/>
-      <c r="B192" s="5"/>
-      <c r="C192" s="5"/>
+      <c r="A192" s="2"/>
+      <c r="B192" s="2"/>
+      <c r="C192" s="2"/>
     </row>
     <row r="193" ht="15" customHeight="1">
-      <c r="A193" s="5"/>
-      <c r="B193" s="5"/>
-      <c r="C193" s="5"/>
+      <c r="A193" s="2"/>
+      <c r="B193" s="2"/>
+      <c r="C193" s="2"/>
     </row>
     <row r="194" ht="15" customHeight="1">
-      <c r="A194" s="5"/>
-      <c r="B194" s="5"/>
-      <c r="C194" s="5"/>
+      <c r="A194" s="2"/>
+      <c r="B194" s="2"/>
+      <c r="C194" s="2"/>
     </row>
     <row r="195" ht="15" customHeight="1">
-      <c r="A195" s="5"/>
-      <c r="B195" s="5"/>
-      <c r="C195" s="5"/>
+      <c r="A195" s="2"/>
+      <c r="B195" s="2"/>
+      <c r="C195" s="2"/>
     </row>
     <row r="196" ht="15" customHeight="1">
-      <c r="A196" s="5"/>
-      <c r="B196" s="5"/>
-      <c r="C196" s="5"/>
+      <c r="A196" s="2"/>
+      <c r="B196" s="2"/>
+      <c r="C196" s="2"/>
     </row>
     <row r="197" ht="15" customHeight="1">
-      <c r="A197" s="5"/>
-      <c r="B197" s="5"/>
-      <c r="C197" s="5"/>
+      <c r="A197" s="2"/>
+      <c r="B197" s="2"/>
+      <c r="C197" s="2"/>
     </row>
     <row r="198" ht="15" customHeight="1">
-      <c r="A198" s="5"/>
-      <c r="B198" s="5"/>
-      <c r="C198" s="5"/>
+      <c r="A198" s="2"/>
+      <c r="B198" s="2"/>
+      <c r="C198" s="2"/>
     </row>
     <row r="199" ht="15" customHeight="1">
-      <c r="A199" s="5"/>
-      <c r="B199" s="5"/>
-      <c r="C199" s="5"/>
+      <c r="A199" s="2"/>
+      <c r="B199" s="2"/>
+      <c r="C199" s="2"/>
     </row>
     <row r="200" ht="15" customHeight="1">
-      <c r="A200" s="5"/>
-      <c r="B200" s="5"/>
-      <c r="C200" s="5"/>
+      <c r="A200" s="2"/>
+      <c r="B200" s="2"/>
+      <c r="C200" s="2"/>
     </row>
     <row r="201" ht="15" customHeight="1">
-      <c r="A201" s="5"/>
-      <c r="B201" s="5"/>
-      <c r="C201" s="5"/>
+      <c r="A201" s="2"/>
+      <c r="B201" s="2"/>
+      <c r="C201" s="2"/>
     </row>
     <row r="202" ht="15" customHeight="1">
-      <c r="A202" s="5"/>
-      <c r="B202" s="5"/>
-      <c r="C202" s="5"/>
+      <c r="A202" s="2"/>
+      <c r="B202" s="2"/>
+      <c r="C202" s="2"/>
     </row>
     <row r="203" ht="15" customHeight="1">
-      <c r="A203" s="5"/>
-      <c r="B203" s="5"/>
-      <c r="C203" s="5"/>
+      <c r="A203" s="2"/>
+      <c r="B203" s="2"/>
+      <c r="C203" s="2"/>
     </row>
     <row r="204" ht="15" customHeight="1">
-      <c r="A204" s="5"/>
-      <c r="B204" s="5"/>
+      <c r="A204" s="2"/>
+      <c r="B204" s="2"/>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>

<commit_message>
Added Scrapper into spreadsheet and Level 2 damage upgrade
Moved Scrapper settings to Excel configuration
Added 1.5x damage boost against Crushers at Level 2
</commit_message>
<xml_diff>
--- a/config/gameplay.xlsx
+++ b/config/gameplay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
   <si>
     <t>enemy_id</t>
   </si>
@@ -96,6 +96,9 @@
     <t>upgrade_health_multiplier</t>
   </si>
   <si>
+    <t>recovery_ms</t>
+  </si>
+  <si>
     <t>shooter</t>
   </si>
   <si>
@@ -112,6 +115,9 @@
   </si>
   <si>
     <t>landmine</t>
+  </si>
+  <si>
+    <t>scrapper</t>
   </si>
   <si>
     <t>setting</t>
@@ -616,7 +622,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{49210968-6DA8-10F8-A4F7-5E35F5FBF9E3}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E5CD549B-EFF8-0848-E254-93B35567AF56}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -823,7 +829,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E5A228F5-2A9E-9C58-0299-9BDDBF263681}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{EB742FF8-4478-FC38-191F-65DE5B700EE1}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -893,10 +899,13 @@
       <c r="P1" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="Q1" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2" s="1">
         <v>300</v>
@@ -943,10 +952,13 @@
       <c r="P2" s="2">
         <v>1</v>
       </c>
+      <c r="Q2" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1">
         <v>300</v>
@@ -993,10 +1005,13 @@
       <c r="P3" s="2">
         <v>1</v>
       </c>
+      <c r="Q3" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2">
         <v>2750</v>
@@ -1043,10 +1058,13 @@
       <c r="P4" s="2">
         <v>1.5</v>
       </c>
+      <c r="Q4" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" s="2">
         <v>300</v>
@@ -1093,10 +1111,13 @@
       <c r="P5" s="2">
         <v>1</v>
       </c>
+      <c r="Q5" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2">
         <v>300</v>
@@ -1143,10 +1164,13 @@
       <c r="P6" s="2">
         <v>1</v>
       </c>
+      <c r="Q6" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" s="2">
         <v>300</v>
@@ -1193,9 +1217,62 @@
       <c r="P7" s="2">
         <v>1</v>
       </c>
+      <c r="Q7" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="2"/>
+      <c r="A8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="4">
+        <v>300</v>
+      </c>
+      <c r="C8" s="4">
+        <v>500</v>
+      </c>
+      <c r="D8" s="4">
+        <v>150</v>
+      </c>
+      <c r="E8" s="4">
+        <v>7500</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4">
+        <v>100</v>
+      </c>
+      <c r="N8" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="O8" s="4">
+        <v>1</v>
+      </c>
+      <c r="P8" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="4">
+        <v>42000</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="M18" s="2"/>
@@ -1213,7 +1290,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{34C27081-BB78-FD58-8FA3-A770F9D16E78}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4CDB60A8-E018-A329-66C6-169B223CBBC3}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1222,15 +1299,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1">
         <v>2000</v>
@@ -1238,7 +1315,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B3" s="1">
         <v>25</v>
@@ -1246,7 +1323,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" s="1">
         <v>7000</v>
@@ -1254,7 +1331,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="1">
         <v>24000</v>
@@ -1262,7 +1339,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" s="1">
         <v>15000</v>
@@ -1270,7 +1347,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B7" s="2">
         <v>0.4</v>
@@ -1278,7 +1355,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B8" s="2">
         <v>20</v>
@@ -1286,7 +1363,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2">
         <v>25</v>
@@ -1294,17 +1371,17 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B10" s="2">
         <v>15000</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="4">
+      <c r="A11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="2">
         <v>0.5</v>
       </c>
     </row>
@@ -1321,7 +1398,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4F8B48F8-4D48-1359-B348-545E7A68C828}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5EB6CDB8-9B1D-A628-A43D-236DCE289FB8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1330,15 +1407,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1">
         <v>500</v>
@@ -1346,7 +1423,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1354,7 +1431,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B4" s="2">
         <v>50</v>
@@ -1373,7 +1450,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{47E5742A-B698-6868-8BC3-10E749DFCCFD}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0F6183FD-56E8-E298-1FF5-7B7C2E65DF08}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T204"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1382,15 +1459,15 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B2" s="1">
         <v>1000</v>
@@ -1398,7 +1475,7 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1">
         <v>1000</v>
@@ -1406,7 +1483,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B4" s="1">
         <v>0.4</v>
@@ -1414,7 +1491,7 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B5" s="1">
         <v>0.2</v>
@@ -1422,7 +1499,7 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B6" s="2">
         <v>0.15</v>
@@ -1430,7 +1507,7 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B7" s="2">
         <v>0.15</v>
@@ -1439,7 +1516,7 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2">
         <v>0.1</v>
@@ -1448,7 +1525,7 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B9" s="2">
         <v>1</v>
@@ -1457,7 +1534,7 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B10" s="2">
         <v>3</v>
@@ -1466,7 +1543,7 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B11" s="2">
         <v>2</v>
@@ -1475,7 +1552,7 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B12" s="2">
         <v>3</v>
@@ -1484,7 +1561,7 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B13" s="2">
         <v>3</v>
@@ -1493,7 +1570,7 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B14" s="2">
         <v>3</v>
@@ -1502,7 +1579,7 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B15" s="2">
         <v>5</v>
@@ -1511,7 +1588,7 @@
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B16" s="2">
         <v>10</v>
@@ -1520,7 +1597,7 @@
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B17" s="2">
         <v>15</v>
@@ -1529,7 +1606,7 @@
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B18" s="2">
         <v>10</v>
@@ -1538,7 +1615,7 @@
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B19" s="2">
         <v>20</v>
@@ -1547,7 +1624,7 @@
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B20" s="2">
         <v>15</v>
@@ -1556,7 +1633,7 @@
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B21" s="2">
         <v>20</v>
@@ -1565,7 +1642,7 @@
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B22" s="2">
         <v>30</v>
@@ -1574,7 +1651,7 @@
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B23" s="2">
         <v>40</v>
@@ -1583,7 +1660,7 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B24" s="2">
         <v>50</v>
@@ -1592,7 +1669,7 @@
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B25" s="2">
         <v>60</v>
@@ -1601,7 +1678,7 @@
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B26" s="2">
         <v>50</v>
@@ -1610,7 +1687,7 @@
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B27" s="2">
         <v>65</v>
@@ -1619,7 +1696,7 @@
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B28" s="2">
         <v>80</v>
@@ -1628,7 +1705,7 @@
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B29" s="2">
         <v>70</v>
@@ -1637,7 +1714,7 @@
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B30" s="2">
         <v>90</v>
@@ -1646,7 +1723,7 @@
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B31" s="2">
         <v>110</v>
@@ -1655,7 +1732,7 @@
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B32" s="2">
         <v>10000</v>
@@ -1664,7 +1741,7 @@
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B33" s="2">
         <v>0.1</v>
@@ -1673,7 +1750,7 @@
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B34" s="2">
         <v>0.05</v>

</xml_diff>